<commit_message>
docs(safari-owner-data): supplier, driver, vehicle and cost sheets; office payment decisions
Owner hub gains six sheets for OPS2-E/F inputs (suppliers, supplier prices,
drivers, vehicles, settlement rules, per-tour costs) with dropdowns and the
27 for-sale tours prefilled. Pending answers record the owner's office
payment methods, deposits, deferred online payment and the approved daily
EUR→EGP rate policy.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/clients/safari-tours-sharm/owner-data/safari-tours-owner-data-hub.xlsx
+++ b/clients/safari-tours-sharm/owner-data/safari-tours-owner-data-hub.xlsx
@@ -18,6 +18,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الأسئلة الشائعة" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="أساس التسويق" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="لوحة المتابعة" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الموردين" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="أسعار الموردين" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="السواقين" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="العربيات" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="التكاليف والتسويات" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="تكاليف الرحلات" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -26,7 +32,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="15">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -108,6 +114,14 @@
       <b val="1"/>
       <color rgb="FF0A2342"/>
       <sz val="15"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF0A2342"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
   <fills count="14">
@@ -229,7 +243,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -437,6 +451,18 @@
     </xf>
     <xf numFmtId="9" fontId="6" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1249,7 +1275,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A35"/>
+  <dimension ref="A1:A42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -1477,6 +1503,48 @@
       <c r="A35" s="63" t="inlineStr">
         <is>
           <t>أي تعديل سعر/سعة/دفع/صلاحية يمر بالـpacket والمراجعة المطلوبة قبل الإنتاج.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>شيتات جديدة (2026-10-05) — للموردين والتكاليف:</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>الموردين — مين بيشتغل معاك وبتحاسبه إزاي وإمتى.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>أسعار الموردين — السعر اللي بتدفعه لكل مورد في كل رحلة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>السواقين والعربيات — مين بيوصّل وبأنهي عربية وبكام.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>التكاليف والتسويات — اعتماد الدفع والعمولات ورد الفلوس.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>تكاليف الرحلات — رسوم الدخول والمرشد والأكل لكل رحلة.</t>
         </is>
       </c>
     </row>
@@ -1491,7 +1559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1649,6 +1717,23 @@
       <c r="C9" t="inlineStr">
         <is>
           <t>تحديث نصوص الرحلات بالإنجليزي في شيت الرحلات من النسخة النهائية (tour-content-drafts.en.json)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>أضاف شيتات الموردين وأسعار الموردين والسواقين والعربيات والتكاليف والتسويات وتكاليف الرحلات — بطلب محمد «اعملها».</t>
         </is>
       </c>
     </row>
@@ -6240,6 +6325,1849 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="30" customWidth="1" min="13" max="13"/>
+    <col width="26" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="48" customHeight="1">
+      <c r="A1" s="80" t="inlineStr">
+        <is>
+          <t>الموردين اللي بينفّذوا الرحلات أو جزء منها (مراكب، كواد، سفاري، غوص، عروض…). سطر لكل مورد. اكتب في الخانات الصفرا بس. الأسعار المتفق عليها تتكتب في شيت «أسعار الموردين».</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="81" t="inlineStr">
+        <is>
+          <t>كود المورد (اكتبه انت: S01, S02…)</t>
+        </is>
+      </c>
+      <c r="B2" s="81" t="inlineStr">
+        <is>
+          <t>اسم المورد / الشركة</t>
+        </is>
+      </c>
+      <c r="C2" s="81" t="inlineStr">
+        <is>
+          <t>نوع الخدمة</t>
+        </is>
+      </c>
+      <c r="D2" s="81" t="inlineStr">
+        <is>
+          <t>الرحلات اللي بيشتغل فيها (أكواد الرحلات)</t>
+        </is>
+      </c>
+      <c r="E2" s="81" t="inlineStr">
+        <is>
+          <t>الشخص المسؤول</t>
+        </is>
+      </c>
+      <c r="F2" s="81" t="inlineStr">
+        <is>
+          <t>موبايل / واتساب الشغل</t>
+        </is>
+      </c>
+      <c r="G2" s="81" t="inlineStr">
+        <is>
+          <t>بتأكد معاه الحجز إزاي؟</t>
+        </is>
+      </c>
+      <c r="H2" s="81" t="inlineStr">
+        <is>
+          <t>لازم تبلّغه قبل الرحلة بكام ساعة؟</t>
+        </is>
+      </c>
+      <c r="I2" s="81" t="inlineStr">
+        <is>
+          <t>بتحاسبه إزاي؟</t>
+        </is>
+      </c>
+      <c r="J2" s="81" t="inlineStr">
+        <is>
+          <t>عملة الحساب</t>
+        </is>
+      </c>
+      <c r="K2" s="81" t="inlineStr">
+        <is>
+          <t>بتحاسبه إمتى؟</t>
+        </is>
+      </c>
+      <c r="L2" s="81" t="inlineStr">
+        <is>
+          <t>بتدفعله إزاي؟</t>
+        </is>
+      </c>
+      <c r="M2" s="81" t="inlineStr">
+        <is>
+          <t>لو الرحلة اتلغت أو العميل ما جاش؟</t>
+        </is>
+      </c>
+      <c r="N2" s="81" t="inlineStr">
+        <is>
+          <t>ملاحظات</t>
+        </is>
+      </c>
+      <c r="O2" s="81" t="inlineStr">
+        <is>
+          <t>الحالة</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="82" t="inlineStr">
+        <is>
+          <t>S01</t>
+        </is>
+      </c>
+      <c r="B3" s="83" t="inlineStr"/>
+      <c r="C3" s="83" t="inlineStr"/>
+      <c r="D3" s="83" t="inlineStr"/>
+      <c r="E3" s="83" t="inlineStr"/>
+      <c r="F3" s="83" t="inlineStr"/>
+      <c r="G3" s="83" t="inlineStr"/>
+      <c r="H3" s="83" t="inlineStr"/>
+      <c r="I3" s="83" t="inlineStr"/>
+      <c r="J3" s="83" t="inlineStr"/>
+      <c r="K3" s="83" t="inlineStr"/>
+      <c r="L3" s="83" t="inlineStr"/>
+      <c r="M3" s="83" t="inlineStr"/>
+      <c r="N3" s="83" t="inlineStr"/>
+      <c r="O3" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="82" t="inlineStr">
+        <is>
+          <t>S02</t>
+        </is>
+      </c>
+      <c r="B4" s="83" t="inlineStr"/>
+      <c r="C4" s="83" t="inlineStr"/>
+      <c r="D4" s="83" t="inlineStr"/>
+      <c r="E4" s="83" t="inlineStr"/>
+      <c r="F4" s="83" t="inlineStr"/>
+      <c r="G4" s="83" t="inlineStr"/>
+      <c r="H4" s="83" t="inlineStr"/>
+      <c r="I4" s="83" t="inlineStr"/>
+      <c r="J4" s="83" t="inlineStr"/>
+      <c r="K4" s="83" t="inlineStr"/>
+      <c r="L4" s="83" t="inlineStr"/>
+      <c r="M4" s="83" t="inlineStr"/>
+      <c r="N4" s="83" t="inlineStr"/>
+      <c r="O4" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="82" t="inlineStr">
+        <is>
+          <t>S03</t>
+        </is>
+      </c>
+      <c r="B5" s="83" t="inlineStr"/>
+      <c r="C5" s="83" t="inlineStr"/>
+      <c r="D5" s="83" t="inlineStr"/>
+      <c r="E5" s="83" t="inlineStr"/>
+      <c r="F5" s="83" t="inlineStr"/>
+      <c r="G5" s="83" t="inlineStr"/>
+      <c r="H5" s="83" t="inlineStr"/>
+      <c r="I5" s="83" t="inlineStr"/>
+      <c r="J5" s="83" t="inlineStr"/>
+      <c r="K5" s="83" t="inlineStr"/>
+      <c r="L5" s="83" t="inlineStr"/>
+      <c r="M5" s="83" t="inlineStr"/>
+      <c r="N5" s="83" t="inlineStr"/>
+      <c r="O5" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="82" t="inlineStr">
+        <is>
+          <t>S04</t>
+        </is>
+      </c>
+      <c r="B6" s="83" t="inlineStr"/>
+      <c r="C6" s="83" t="inlineStr"/>
+      <c r="D6" s="83" t="inlineStr"/>
+      <c r="E6" s="83" t="inlineStr"/>
+      <c r="F6" s="83" t="inlineStr"/>
+      <c r="G6" s="83" t="inlineStr"/>
+      <c r="H6" s="83" t="inlineStr"/>
+      <c r="I6" s="83" t="inlineStr"/>
+      <c r="J6" s="83" t="inlineStr"/>
+      <c r="K6" s="83" t="inlineStr"/>
+      <c r="L6" s="83" t="inlineStr"/>
+      <c r="M6" s="83" t="inlineStr"/>
+      <c r="N6" s="83" t="inlineStr"/>
+      <c r="O6" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="82" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="B7" s="83" t="inlineStr"/>
+      <c r="C7" s="83" t="inlineStr"/>
+      <c r="D7" s="83" t="inlineStr"/>
+      <c r="E7" s="83" t="inlineStr"/>
+      <c r="F7" s="83" t="inlineStr"/>
+      <c r="G7" s="83" t="inlineStr"/>
+      <c r="H7" s="83" t="inlineStr"/>
+      <c r="I7" s="83" t="inlineStr"/>
+      <c r="J7" s="83" t="inlineStr"/>
+      <c r="K7" s="83" t="inlineStr"/>
+      <c r="L7" s="83" t="inlineStr"/>
+      <c r="M7" s="83" t="inlineStr"/>
+      <c r="N7" s="83" t="inlineStr"/>
+      <c r="O7" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="82" t="inlineStr">
+        <is>
+          <t>S06</t>
+        </is>
+      </c>
+      <c r="B8" s="83" t="inlineStr"/>
+      <c r="C8" s="83" t="inlineStr"/>
+      <c r="D8" s="83" t="inlineStr"/>
+      <c r="E8" s="83" t="inlineStr"/>
+      <c r="F8" s="83" t="inlineStr"/>
+      <c r="G8" s="83" t="inlineStr"/>
+      <c r="H8" s="83" t="inlineStr"/>
+      <c r="I8" s="83" t="inlineStr"/>
+      <c r="J8" s="83" t="inlineStr"/>
+      <c r="K8" s="83" t="inlineStr"/>
+      <c r="L8" s="83" t="inlineStr"/>
+      <c r="M8" s="83" t="inlineStr"/>
+      <c r="N8" s="83" t="inlineStr"/>
+      <c r="O8" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="82" t="inlineStr">
+        <is>
+          <t>S07</t>
+        </is>
+      </c>
+      <c r="B9" s="83" t="inlineStr"/>
+      <c r="C9" s="83" t="inlineStr"/>
+      <c r="D9" s="83" t="inlineStr"/>
+      <c r="E9" s="83" t="inlineStr"/>
+      <c r="F9" s="83" t="inlineStr"/>
+      <c r="G9" s="83" t="inlineStr"/>
+      <c r="H9" s="83" t="inlineStr"/>
+      <c r="I9" s="83" t="inlineStr"/>
+      <c r="J9" s="83" t="inlineStr"/>
+      <c r="K9" s="83" t="inlineStr"/>
+      <c r="L9" s="83" t="inlineStr"/>
+      <c r="M9" s="83" t="inlineStr"/>
+      <c r="N9" s="83" t="inlineStr"/>
+      <c r="O9" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="82" t="inlineStr">
+        <is>
+          <t>S08</t>
+        </is>
+      </c>
+      <c r="B10" s="83" t="inlineStr"/>
+      <c r="C10" s="83" t="inlineStr"/>
+      <c r="D10" s="83" t="inlineStr"/>
+      <c r="E10" s="83" t="inlineStr"/>
+      <c r="F10" s="83" t="inlineStr"/>
+      <c r="G10" s="83" t="inlineStr"/>
+      <c r="H10" s="83" t="inlineStr"/>
+      <c r="I10" s="83" t="inlineStr"/>
+      <c r="J10" s="83" t="inlineStr"/>
+      <c r="K10" s="83" t="inlineStr"/>
+      <c r="L10" s="83" t="inlineStr"/>
+      <c r="M10" s="83" t="inlineStr"/>
+      <c r="N10" s="83" t="inlineStr"/>
+      <c r="O10" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="82" t="inlineStr">
+        <is>
+          <t>S09</t>
+        </is>
+      </c>
+      <c r="B11" s="83" t="inlineStr"/>
+      <c r="C11" s="83" t="inlineStr"/>
+      <c r="D11" s="83" t="inlineStr"/>
+      <c r="E11" s="83" t="inlineStr"/>
+      <c r="F11" s="83" t="inlineStr"/>
+      <c r="G11" s="83" t="inlineStr"/>
+      <c r="H11" s="83" t="inlineStr"/>
+      <c r="I11" s="83" t="inlineStr"/>
+      <c r="J11" s="83" t="inlineStr"/>
+      <c r="K11" s="83" t="inlineStr"/>
+      <c r="L11" s="83" t="inlineStr"/>
+      <c r="M11" s="83" t="inlineStr"/>
+      <c r="N11" s="83" t="inlineStr"/>
+      <c r="O11" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="82" t="inlineStr">
+        <is>
+          <t>S10</t>
+        </is>
+      </c>
+      <c r="B12" s="83" t="inlineStr"/>
+      <c r="C12" s="83" t="inlineStr"/>
+      <c r="D12" s="83" t="inlineStr"/>
+      <c r="E12" s="83" t="inlineStr"/>
+      <c r="F12" s="83" t="inlineStr"/>
+      <c r="G12" s="83" t="inlineStr"/>
+      <c r="H12" s="83" t="inlineStr"/>
+      <c r="I12" s="83" t="inlineStr"/>
+      <c r="J12" s="83" t="inlineStr"/>
+      <c r="K12" s="83" t="inlineStr"/>
+      <c r="L12" s="83" t="inlineStr"/>
+      <c r="M12" s="83" t="inlineStr"/>
+      <c r="N12" s="83" t="inlineStr"/>
+      <c r="O12" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="82" t="inlineStr">
+        <is>
+          <t>S11</t>
+        </is>
+      </c>
+      <c r="B13" s="83" t="inlineStr"/>
+      <c r="C13" s="83" t="inlineStr"/>
+      <c r="D13" s="83" t="inlineStr"/>
+      <c r="E13" s="83" t="inlineStr"/>
+      <c r="F13" s="83" t="inlineStr"/>
+      <c r="G13" s="83" t="inlineStr"/>
+      <c r="H13" s="83" t="inlineStr"/>
+      <c r="I13" s="83" t="inlineStr"/>
+      <c r="J13" s="83" t="inlineStr"/>
+      <c r="K13" s="83" t="inlineStr"/>
+      <c r="L13" s="83" t="inlineStr"/>
+      <c r="M13" s="83" t="inlineStr"/>
+      <c r="N13" s="83" t="inlineStr"/>
+      <c r="O13" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="82" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="B14" s="83" t="inlineStr"/>
+      <c r="C14" s="83" t="inlineStr"/>
+      <c r="D14" s="83" t="inlineStr"/>
+      <c r="E14" s="83" t="inlineStr"/>
+      <c r="F14" s="83" t="inlineStr"/>
+      <c r="G14" s="83" t="inlineStr"/>
+      <c r="H14" s="83" t="inlineStr"/>
+      <c r="I14" s="83" t="inlineStr"/>
+      <c r="J14" s="83" t="inlineStr"/>
+      <c r="K14" s="83" t="inlineStr"/>
+      <c r="L14" s="83" t="inlineStr"/>
+      <c r="M14" s="83" t="inlineStr"/>
+      <c r="N14" s="83" t="inlineStr"/>
+      <c r="O14" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="82" t="inlineStr">
+        <is>
+          <t>S13</t>
+        </is>
+      </c>
+      <c r="B15" s="83" t="inlineStr"/>
+      <c r="C15" s="83" t="inlineStr"/>
+      <c r="D15" s="83" t="inlineStr"/>
+      <c r="E15" s="83" t="inlineStr"/>
+      <c r="F15" s="83" t="inlineStr"/>
+      <c r="G15" s="83" t="inlineStr"/>
+      <c r="H15" s="83" t="inlineStr"/>
+      <c r="I15" s="83" t="inlineStr"/>
+      <c r="J15" s="83" t="inlineStr"/>
+      <c r="K15" s="83" t="inlineStr"/>
+      <c r="L15" s="83" t="inlineStr"/>
+      <c r="M15" s="83" t="inlineStr"/>
+      <c r="N15" s="83" t="inlineStr"/>
+      <c r="O15" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="82" t="inlineStr">
+        <is>
+          <t>S14</t>
+        </is>
+      </c>
+      <c r="B16" s="83" t="inlineStr"/>
+      <c r="C16" s="83" t="inlineStr"/>
+      <c r="D16" s="83" t="inlineStr"/>
+      <c r="E16" s="83" t="inlineStr"/>
+      <c r="F16" s="83" t="inlineStr"/>
+      <c r="G16" s="83" t="inlineStr"/>
+      <c r="H16" s="83" t="inlineStr"/>
+      <c r="I16" s="83" t="inlineStr"/>
+      <c r="J16" s="83" t="inlineStr"/>
+      <c r="K16" s="83" t="inlineStr"/>
+      <c r="L16" s="83" t="inlineStr"/>
+      <c r="M16" s="83" t="inlineStr"/>
+      <c r="N16" s="83" t="inlineStr"/>
+      <c r="O16" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="82" t="inlineStr">
+        <is>
+          <t>S15</t>
+        </is>
+      </c>
+      <c r="B17" s="83" t="inlineStr"/>
+      <c r="C17" s="83" t="inlineStr"/>
+      <c r="D17" s="83" t="inlineStr"/>
+      <c r="E17" s="83" t="inlineStr"/>
+      <c r="F17" s="83" t="inlineStr"/>
+      <c r="G17" s="83" t="inlineStr"/>
+      <c r="H17" s="83" t="inlineStr"/>
+      <c r="I17" s="83" t="inlineStr"/>
+      <c r="J17" s="83" t="inlineStr"/>
+      <c r="K17" s="83" t="inlineStr"/>
+      <c r="L17" s="83" t="inlineStr"/>
+      <c r="M17" s="83" t="inlineStr"/>
+      <c r="N17" s="83" t="inlineStr"/>
+      <c r="O17" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:O1"/>
+  </mergeCells>
+  <dataValidations count="7">
+    <dataValidation sqref="C3:C17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"مراكب,كواد/باجي/سفاري,غوص/سنوركل,عروض وترفيه,نقل/عربيات,مرشدين,طيران/رحلات بعيدة,أخرى"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G3:G17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"واتساب,تليفون,إيميل,بيجي المكتب"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I3:I17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"سعر ثابت للرحلة,لكل فرد,لكل وحدة (باجي/مركب/عربية),نسبة من سعر البيع"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J3:J17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"جنيه,يورو,دولار"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K3:K17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"بعد كل رحلة,آخر الأسبوع,آخر الشهر,غير كده (اكتب في الملاحظات)"</formula1>
+    </dataValidation>
+    <dataValidation sqref="L3:L17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"كاش,تحويل بنكي,إنستاباي,محفظة إلكترونية"</formula1>
+    </dataValidation>
+    <dataValidation sqref="O3:O17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"ناقص,اتملى,محتاج مراجعة,مش محتاجينه"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="48" customHeight="1">
+      <c r="A1" s="80" t="inlineStr">
+        <is>
+          <t>السعر اللي بتدفعه للمورد (مش سعر البيع). سطر لكل رحلة مع كل مورد — لو الرحلة ليها أكتر من مورد، اعمل نسخة من السطر. املا العمود اللي يناسب طريقة الحساب بس.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="81" t="inlineStr">
+        <is>
+          <t>كود الرحلة</t>
+        </is>
+      </c>
+      <c r="B2" s="81" t="inlineStr">
+        <is>
+          <t>كود المورد (من شيت الموردين)</t>
+        </is>
+      </c>
+      <c r="C2" s="81" t="inlineStr">
+        <is>
+          <t>سعر البالغ</t>
+        </is>
+      </c>
+      <c r="D2" s="81" t="inlineStr">
+        <is>
+          <t>سعر الطفل</t>
+        </is>
+      </c>
+      <c r="E2" s="81" t="inlineStr">
+        <is>
+          <t>سعر الوحدة (باجي/مركب/عربية)</t>
+        </is>
+      </c>
+      <c r="F2" s="81" t="inlineStr">
+        <is>
+          <t>نسبة من سعر البيع %</t>
+        </is>
+      </c>
+      <c r="G2" s="81" t="inlineStr">
+        <is>
+          <t>العملة</t>
+        </is>
+      </c>
+      <c r="H2" s="81" t="inlineStr">
+        <is>
+          <t>الموسم</t>
+        </is>
+      </c>
+      <c r="I2" s="81" t="inlineStr">
+        <is>
+          <t>ساري من (تاريخ)</t>
+        </is>
+      </c>
+      <c r="J2" s="81" t="inlineStr">
+        <is>
+          <t>ساري لحد (تاريخ)</t>
+        </is>
+      </c>
+      <c r="K2" s="81" t="inlineStr">
+        <is>
+          <t>ملاحظات</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="82" t="inlineStr">
+        <is>
+          <t>super-safari-adventure</t>
+        </is>
+      </c>
+      <c r="B3" s="83" t="inlineStr"/>
+      <c r="C3" s="83" t="inlineStr"/>
+      <c r="D3" s="83" t="inlineStr"/>
+      <c r="E3" s="83" t="inlineStr"/>
+      <c r="F3" s="83" t="inlineStr"/>
+      <c r="G3" s="83" t="inlineStr"/>
+      <c r="H3" s="83" t="inlineStr">
+        <is>
+          <t>كل السنة</t>
+        </is>
+      </c>
+      <c r="I3" s="83" t="inlineStr"/>
+      <c r="J3" s="83" t="inlineStr"/>
+      <c r="K3" s="83" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="82" t="inlineStr">
+        <is>
+          <t>sunset-quad-bike</t>
+        </is>
+      </c>
+      <c r="B4" s="83" t="inlineStr"/>
+      <c r="C4" s="83" t="inlineStr"/>
+      <c r="D4" s="83" t="inlineStr"/>
+      <c r="E4" s="83" t="inlineStr"/>
+      <c r="F4" s="83" t="inlineStr"/>
+      <c r="G4" s="83" t="inlineStr"/>
+      <c r="H4" s="83" t="inlineStr">
+        <is>
+          <t>كل السنة</t>
+        </is>
+      </c>
+      <c r="I4" s="83" t="inlineStr"/>
+      <c r="J4" s="83" t="inlineStr"/>
+      <c r="K4" s="83" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="82" t="inlineStr">
+        <is>
+          <t>double-buggy-camel-ride</t>
+        </is>
+      </c>
+      <c r="B5" s="83" t="inlineStr"/>
+      <c r="C5" s="83" t="inlineStr"/>
+      <c r="D5" s="83" t="inlineStr"/>
+      <c r="E5" s="83" t="inlineStr"/>
+      <c r="F5" s="83" t="inlineStr"/>
+      <c r="G5" s="83" t="inlineStr"/>
+      <c r="H5" s="83" t="inlineStr">
+        <is>
+          <t>كل السنة</t>
+        </is>
+      </c>
+      <c r="I5" s="83" t="inlineStr"/>
+      <c r="J5" s="83" t="inlineStr"/>
+      <c r="K5" s="83" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="82" t="inlineStr">
+        <is>
+          <t>bedouin-dinner-camel-ride</t>
+        </is>
+      </c>
+      <c r="B6" s="83" t="inlineStr"/>
+      <c r="C6" s="83" t="inlineStr"/>
+      <c r="D6" s="83" t="inlineStr"/>
+      <c r="E6" s="83" t="inlineStr"/>
+      <c r="F6" s="83" t="inlineStr"/>
+      <c r="G6" s="83" t="inlineStr"/>
+      <c r="H6" s="83" t="inlineStr">
+        <is>
+          <t>كل السنة</t>
+        </is>
+      </c>
+      <c r="I6" s="83" t="inlineStr"/>
+      <c r="J6" s="83" t="inlineStr"/>
+      <c r="K6" s="83" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="82" t="inlineStr">
+        <is>
+          <t>dahab-colored-canyon</t>
+        </is>
+      </c>
+      <c r="B7" s="83" t="inlineStr"/>
+      <c r="C7" s="83" t="inlineStr"/>
+      <c r="D7" s="83" t="inlineStr"/>
+      <c r="E7" s="83" t="inlineStr"/>
+      <c r="F7" s="83" t="inlineStr"/>
+      <c r="G7" s="83" t="inlineStr"/>
+      <c r="H7" s="83" t="inlineStr">
+        <is>
+          <t>كل السنة</t>
+        </is>
+      </c>
+      <c r="I7" s="83" t="inlineStr"/>
+      <c r="J7" s="83" t="inlineStr"/>
+      <c r="K7" s="83" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="82" t="inlineStr">
+        <is>
+          <t>camel-horse-ride</t>
+        </is>
+      </c>
+      <c r="B8" s="83" t="inlineStr"/>
+      <c r="C8" s="83" t="inlineStr"/>
+      <c r="D8" s="83" t="inlineStr"/>
+      <c r="E8" s="83" t="inlineStr"/>
+      <c r="F8" s="83" t="inlineStr"/>
+      <c r="G8" s="83" t="inlineStr"/>
+      <c r="H8" s="83" t="inlineStr">
+        <is>
+          <t>كل السنة</t>
+        </is>
+      </c>
+      <c r="I8" s="83" t="inlineStr"/>
+      <c r="J8" s="83" t="inlineStr"/>
+      <c r="K8" s="83" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="82" t="inlineStr">
+        <is>
+          <t>ras-mohamed-white-island-boat</t>
+        </is>
+      </c>
+      <c r="B9" s="83" t="inlineStr"/>
+      <c r="C9" s="83" t="inlineStr"/>
+      <c r="D9" s="83" t="inlineStr"/>
+      <c r="E9" s="83" t="inlineStr"/>
+      <c r="F9" s="83" t="inlineStr"/>
+      <c r="G9" s="83" t="inlineStr"/>
+      <c r="H9" s="83" t="inlineStr">
+        <is>
+          <t>كل السنة</t>
+        </is>
+      </c>
+      <c r="I9" s="83" t="inlineStr"/>
+      <c r="J9" s="83" t="inlineStr"/>
+      <c r="K9" s="83" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="82" t="inlineStr">
+        <is>
+          <t>evening-cruise</t>
+        </is>
+      </c>
+      <c r="B10" s="83" t="inlineStr"/>
+      <c r="C10" s="83" t="inlineStr"/>
+      <c r="D10" s="83" t="inlineStr"/>
+      <c r="E10" s="83" t="inlineStr"/>
+      <c r="F10" s="83" t="inlineStr"/>
+      <c r="G10" s="83" t="inlineStr"/>
+      <c r="H10" s="83" t="inlineStr">
+        <is>
+          <t>كل السنة</t>
+        </is>
+      </c>
+      <c r="I10" s="83" t="inlineStr"/>
+      <c r="J10" s="83" t="inlineStr"/>
+      <c r="K10" s="83" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="82" t="inlineStr">
+        <is>
+          <t>glass-bottom-boat</t>
+        </is>
+      </c>
+      <c r="B11" s="83" t="inlineStr"/>
+      <c r="C11" s="83" t="inlineStr"/>
+      <c r="D11" s="83" t="inlineStr"/>
+      <c r="E11" s="83" t="inlineStr"/>
+      <c r="F11" s="83" t="inlineStr"/>
+      <c r="G11" s="83" t="inlineStr"/>
+      <c r="H11" s="83" t="inlineStr">
+        <is>
+          <t>كل السنة</t>
+        </is>
+      </c>
+      <c r="I11" s="83" t="inlineStr"/>
+      <c r="J11" s="83" t="inlineStr"/>
+      <c r="K11" s="83" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="82" t="inlineStr">
+        <is>
+          <t>diving-course</t>
+        </is>
+      </c>
+      <c r="B12" s="83" t="inlineStr"/>
+      <c r="C12" s="83" t="inlineStr"/>
+      <c r="D12" s="83" t="inlineStr"/>
+      <c r="E12" s="83" t="inlineStr"/>
+      <c r="F12" s="83" t="inlineStr"/>
+      <c r="G12" s="83" t="inlineStr"/>
+      <c r="H12" s="83" t="inlineStr">
+        <is>
+          <t>كل السنة</t>
+        </is>
+      </c>
+      <c r="I12" s="83" t="inlineStr"/>
+      <c r="J12" s="83" t="inlineStr"/>
+      <c r="K12" s="83" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="82" t="inlineStr">
+        <is>
+          <t>sinai-dream-sailboat</t>
+        </is>
+      </c>
+      <c r="B13" s="83" t="inlineStr"/>
+      <c r="C13" s="83" t="inlineStr"/>
+      <c r="D13" s="83" t="inlineStr"/>
+      <c r="E13" s="83" t="inlineStr"/>
+      <c r="F13" s="83" t="inlineStr"/>
+      <c r="G13" s="83" t="inlineStr"/>
+      <c r="H13" s="83" t="inlineStr">
+        <is>
+          <t>كل السنة</t>
+        </is>
+      </c>
+      <c r="I13" s="83" t="inlineStr"/>
+      <c r="J13" s="83" t="inlineStr"/>
+      <c r="K13" s="83" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="82" t="inlineStr">
+        <is>
+          <t>ras-mohamed-by-bus</t>
+        </is>
+      </c>
+      <c r="B14" s="83" t="inlineStr"/>
+      <c r="C14" s="83" t="inlineStr"/>
+      <c r="D14" s="83" t="inlineStr"/>
+      <c r="E14" s="83" t="inlineStr"/>
+      <c r="F14" s="83" t="inlineStr"/>
+      <c r="G14" s="83" t="inlineStr"/>
+      <c r="H14" s="83" t="inlineStr">
+        <is>
+          <t>كل السنة</t>
+        </is>
+      </c>
+      <c r="I14" s="83" t="inlineStr"/>
+      <c r="J14" s="83" t="inlineStr"/>
+      <c r="K14" s="83" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="82" t="inlineStr">
+        <is>
+          <t>banana-boat</t>
+        </is>
+      </c>
+      <c r="B15" s="83" t="inlineStr"/>
+      <c r="C15" s="83" t="inlineStr"/>
+      <c r="D15" s="83" t="inlineStr"/>
+      <c r="E15" s="83" t="inlineStr"/>
+      <c r="F15" s="83" t="inlineStr"/>
+      <c r="G15" s="83" t="inlineStr"/>
+      <c r="H15" s="83" t="inlineStr">
+        <is>
+          <t>كل السنة</t>
+        </is>
+      </c>
+      <c r="I15" s="83" t="inlineStr"/>
+      <c r="J15" s="83" t="inlineStr"/>
+      <c r="K15" s="83" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="82" t="inlineStr">
+        <is>
+          <t>parasailing-adventure</t>
+        </is>
+      </c>
+      <c r="B16" s="83" t="inlineStr"/>
+      <c r="C16" s="83" t="inlineStr"/>
+      <c r="D16" s="83" t="inlineStr"/>
+      <c r="E16" s="83" t="inlineStr"/>
+      <c r="F16" s="83" t="inlineStr"/>
+      <c r="G16" s="83" t="inlineStr"/>
+      <c r="H16" s="83" t="inlineStr">
+        <is>
+          <t>كل السنة</t>
+        </is>
+      </c>
+      <c r="I16" s="83" t="inlineStr"/>
+      <c r="J16" s="83" t="inlineStr"/>
+      <c r="K16" s="83" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="82" t="inlineStr">
+        <is>
+          <t>speed-boat-adventure</t>
+        </is>
+      </c>
+      <c r="B17" s="83" t="inlineStr"/>
+      <c r="C17" s="83" t="inlineStr"/>
+      <c r="D17" s="83" t="inlineStr"/>
+      <c r="E17" s="83" t="inlineStr"/>
+      <c r="F17" s="83" t="inlineStr"/>
+      <c r="G17" s="83" t="inlineStr"/>
+      <c r="H17" s="83" t="inlineStr">
+        <is>
+          <t>كل السنة</t>
+        </is>
+      </c>
+      <c r="I17" s="83" t="inlineStr"/>
+      <c r="J17" s="83" t="inlineStr"/>
+      <c r="K17" s="83" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="82" t="inlineStr">
+        <is>
+          <t>submarine</t>
+        </is>
+      </c>
+      <c r="B18" s="83" t="inlineStr"/>
+      <c r="C18" s="83" t="inlineStr"/>
+      <c r="D18" s="83" t="inlineStr"/>
+      <c r="E18" s="83" t="inlineStr"/>
+      <c r="F18" s="83" t="inlineStr"/>
+      <c r="G18" s="83" t="inlineStr"/>
+      <c r="H18" s="83" t="inlineStr">
+        <is>
+          <t>كل السنة</t>
+        </is>
+      </c>
+      <c r="I18" s="83" t="inlineStr"/>
+      <c r="J18" s="83" t="inlineStr"/>
+      <c r="K18" s="83" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="82" t="inlineStr">
+        <is>
+          <t>tiran-island-boat-trip</t>
+        </is>
+      </c>
+      <c r="B19" s="83" t="inlineStr"/>
+      <c r="C19" s="83" t="inlineStr"/>
+      <c r="D19" s="83" t="inlineStr"/>
+      <c r="E19" s="83" t="inlineStr"/>
+      <c r="F19" s="83" t="inlineStr"/>
+      <c r="G19" s="83" t="inlineStr"/>
+      <c r="H19" s="83" t="inlineStr">
+        <is>
+          <t>كل السنة</t>
+        </is>
+      </c>
+      <c r="I19" s="83" t="inlineStr"/>
+      <c r="J19" s="83" t="inlineStr"/>
+      <c r="K19" s="83" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="82" t="inlineStr">
+        <is>
+          <t>tube-boat</t>
+        </is>
+      </c>
+      <c r="B20" s="83" t="inlineStr"/>
+      <c r="C20" s="83" t="inlineStr"/>
+      <c r="D20" s="83" t="inlineStr"/>
+      <c r="E20" s="83" t="inlineStr"/>
+      <c r="F20" s="83" t="inlineStr"/>
+      <c r="G20" s="83" t="inlineStr"/>
+      <c r="H20" s="83" t="inlineStr">
+        <is>
+          <t>كل السنة</t>
+        </is>
+      </c>
+      <c r="I20" s="83" t="inlineStr"/>
+      <c r="J20" s="83" t="inlineStr"/>
+      <c r="K20" s="83" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="82" t="inlineStr">
+        <is>
+          <t>cairo-by-bus</t>
+        </is>
+      </c>
+      <c r="B21" s="83" t="inlineStr"/>
+      <c r="C21" s="83" t="inlineStr"/>
+      <c r="D21" s="83" t="inlineStr"/>
+      <c r="E21" s="83" t="inlineStr"/>
+      <c r="F21" s="83" t="inlineStr"/>
+      <c r="G21" s="83" t="inlineStr"/>
+      <c r="H21" s="83" t="inlineStr">
+        <is>
+          <t>كل السنة</t>
+        </is>
+      </c>
+      <c r="I21" s="83" t="inlineStr"/>
+      <c r="J21" s="83" t="inlineStr"/>
+      <c r="K21" s="83" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="82" t="inlineStr">
+        <is>
+          <t>cairo-by-plane</t>
+        </is>
+      </c>
+      <c r="B22" s="83" t="inlineStr"/>
+      <c r="C22" s="83" t="inlineStr"/>
+      <c r="D22" s="83" t="inlineStr"/>
+      <c r="E22" s="83" t="inlineStr"/>
+      <c r="F22" s="83" t="inlineStr"/>
+      <c r="G22" s="83" t="inlineStr"/>
+      <c r="H22" s="83" t="inlineStr">
+        <is>
+          <t>كل السنة</t>
+        </is>
+      </c>
+      <c r="I22" s="83" t="inlineStr"/>
+      <c r="J22" s="83" t="inlineStr"/>
+      <c r="K22" s="83" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="82" t="inlineStr">
+        <is>
+          <t>mount-sinai-st-catherine</t>
+        </is>
+      </c>
+      <c r="B23" s="83" t="inlineStr"/>
+      <c r="C23" s="83" t="inlineStr"/>
+      <c r="D23" s="83" t="inlineStr"/>
+      <c r="E23" s="83" t="inlineStr"/>
+      <c r="F23" s="83" t="inlineStr"/>
+      <c r="G23" s="83" t="inlineStr"/>
+      <c r="H23" s="83" t="inlineStr">
+        <is>
+          <t>كل السنة</t>
+        </is>
+      </c>
+      <c r="I23" s="83" t="inlineStr"/>
+      <c r="J23" s="83" t="inlineStr"/>
+      <c r="K23" s="83" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="82" t="inlineStr">
+        <is>
+          <t>luxor-by-plane</t>
+        </is>
+      </c>
+      <c r="B24" s="83" t="inlineStr"/>
+      <c r="C24" s="83" t="inlineStr"/>
+      <c r="D24" s="83" t="inlineStr"/>
+      <c r="E24" s="83" t="inlineStr"/>
+      <c r="F24" s="83" t="inlineStr"/>
+      <c r="G24" s="83" t="inlineStr"/>
+      <c r="H24" s="83" t="inlineStr">
+        <is>
+          <t>كل السنة</t>
+        </is>
+      </c>
+      <c r="I24" s="83" t="inlineStr"/>
+      <c r="J24" s="83" t="inlineStr"/>
+      <c r="K24" s="83" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="82" t="inlineStr">
+        <is>
+          <t>st-catherine-dahab</t>
+        </is>
+      </c>
+      <c r="B25" s="83" t="inlineStr"/>
+      <c r="C25" s="83" t="inlineStr"/>
+      <c r="D25" s="83" t="inlineStr"/>
+      <c r="E25" s="83" t="inlineStr"/>
+      <c r="F25" s="83" t="inlineStr"/>
+      <c r="G25" s="83" t="inlineStr"/>
+      <c r="H25" s="83" t="inlineStr">
+        <is>
+          <t>كل السنة</t>
+        </is>
+      </c>
+      <c r="I25" s="83" t="inlineStr"/>
+      <c r="J25" s="83" t="inlineStr"/>
+      <c r="K25" s="83" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="82" t="inlineStr">
+        <is>
+          <t>turkish-bath</t>
+        </is>
+      </c>
+      <c r="B26" s="83" t="inlineStr"/>
+      <c r="C26" s="83" t="inlineStr"/>
+      <c r="D26" s="83" t="inlineStr"/>
+      <c r="E26" s="83" t="inlineStr"/>
+      <c r="F26" s="83" t="inlineStr"/>
+      <c r="G26" s="83" t="inlineStr"/>
+      <c r="H26" s="83" t="inlineStr">
+        <is>
+          <t>كل السنة</t>
+        </is>
+      </c>
+      <c r="I26" s="83" t="inlineStr"/>
+      <c r="J26" s="83" t="inlineStr"/>
+      <c r="K26" s="83" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="82" t="inlineStr">
+        <is>
+          <t>dolphin-show</t>
+        </is>
+      </c>
+      <c r="B27" s="83" t="inlineStr"/>
+      <c r="C27" s="83" t="inlineStr"/>
+      <c r="D27" s="83" t="inlineStr"/>
+      <c r="E27" s="83" t="inlineStr"/>
+      <c r="F27" s="83" t="inlineStr"/>
+      <c r="G27" s="83" t="inlineStr"/>
+      <c r="H27" s="83" t="inlineStr">
+        <is>
+          <t>كل السنة</t>
+        </is>
+      </c>
+      <c r="I27" s="83" t="inlineStr"/>
+      <c r="J27" s="83" t="inlineStr"/>
+      <c r="K27" s="83" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="82" t="inlineStr">
+        <is>
+          <t>swimming-with-dolphins</t>
+        </is>
+      </c>
+      <c r="B28" s="83" t="inlineStr"/>
+      <c r="C28" s="83" t="inlineStr"/>
+      <c r="D28" s="83" t="inlineStr"/>
+      <c r="E28" s="83" t="inlineStr"/>
+      <c r="F28" s="83" t="inlineStr"/>
+      <c r="G28" s="83" t="inlineStr"/>
+      <c r="H28" s="83" t="inlineStr">
+        <is>
+          <t>كل السنة</t>
+        </is>
+      </c>
+      <c r="I28" s="83" t="inlineStr"/>
+      <c r="J28" s="83" t="inlineStr"/>
+      <c r="K28" s="83" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="82" t="inlineStr">
+        <is>
+          <t>sharm-airport-transfer</t>
+        </is>
+      </c>
+      <c r="B29" s="83" t="inlineStr"/>
+      <c r="C29" s="83" t="inlineStr"/>
+      <c r="D29" s="83" t="inlineStr"/>
+      <c r="E29" s="83" t="inlineStr"/>
+      <c r="F29" s="83" t="inlineStr"/>
+      <c r="G29" s="83" t="inlineStr"/>
+      <c r="H29" s="83" t="inlineStr">
+        <is>
+          <t>كل السنة</t>
+        </is>
+      </c>
+      <c r="I29" s="83" t="inlineStr"/>
+      <c r="J29" s="83" t="inlineStr"/>
+      <c r="K29" s="83" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:K1"/>
+  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="G3:G29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"جنيه,يورو,دولار"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H3:H29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"كل السنة,موسم عالي,موسم عادي"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="48" customHeight="1">
+      <c r="A1" s="80" t="inlineStr">
+        <is>
+          <t>السواقين اللي بيوصّلوا العملاء. ممنوع تكتب رقم بطاقة أو بيانات شخصية زيادة — الاسم وموبايل الشغل كفاية.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="81" t="inlineStr">
+        <is>
+          <t>كود السواق (D01…)</t>
+        </is>
+      </c>
+      <c r="B2" s="81" t="inlineStr">
+        <is>
+          <t>الاسم</t>
+        </is>
+      </c>
+      <c r="C2" s="81" t="inlineStr">
+        <is>
+          <t>موبايل الشغل (اختياري)</t>
+        </is>
+      </c>
+      <c r="D2" s="81" t="inlineStr">
+        <is>
+          <t>نوع التعاقد</t>
+        </is>
+      </c>
+      <c r="E2" s="81" t="inlineStr">
+        <is>
+          <t>الأجر</t>
+        </is>
+      </c>
+      <c r="F2" s="81" t="inlineStr">
+        <is>
+          <t>على أساس</t>
+        </is>
+      </c>
+      <c r="G2" s="81" t="inlineStr">
+        <is>
+          <t>العملة</t>
+        </is>
+      </c>
+      <c r="H2" s="81" t="inlineStr">
+        <is>
+          <t>الرخصة سارية لحد</t>
+        </is>
+      </c>
+      <c r="I2" s="81" t="inlineStr">
+        <is>
+          <t>يسوق أنهي عربيات</t>
+        </is>
+      </c>
+      <c r="J2" s="81" t="inlineStr">
+        <is>
+          <t>ملاحظات</t>
+        </is>
+      </c>
+      <c r="K2" s="81" t="inlineStr">
+        <is>
+          <t>الحالة</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="82" t="inlineStr">
+        <is>
+          <t>D01</t>
+        </is>
+      </c>
+      <c r="B3" s="83" t="inlineStr"/>
+      <c r="C3" s="83" t="inlineStr"/>
+      <c r="D3" s="83" t="inlineStr"/>
+      <c r="E3" s="83" t="inlineStr"/>
+      <c r="F3" s="83" t="inlineStr"/>
+      <c r="G3" s="83" t="inlineStr"/>
+      <c r="H3" s="83" t="inlineStr"/>
+      <c r="I3" s="83" t="inlineStr"/>
+      <c r="J3" s="83" t="inlineStr"/>
+      <c r="K3" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="82" t="inlineStr">
+        <is>
+          <t>D02</t>
+        </is>
+      </c>
+      <c r="B4" s="83" t="inlineStr"/>
+      <c r="C4" s="83" t="inlineStr"/>
+      <c r="D4" s="83" t="inlineStr"/>
+      <c r="E4" s="83" t="inlineStr"/>
+      <c r="F4" s="83" t="inlineStr"/>
+      <c r="G4" s="83" t="inlineStr"/>
+      <c r="H4" s="83" t="inlineStr"/>
+      <c r="I4" s="83" t="inlineStr"/>
+      <c r="J4" s="83" t="inlineStr"/>
+      <c r="K4" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="82" t="inlineStr">
+        <is>
+          <t>D03</t>
+        </is>
+      </c>
+      <c r="B5" s="83" t="inlineStr"/>
+      <c r="C5" s="83" t="inlineStr"/>
+      <c r="D5" s="83" t="inlineStr"/>
+      <c r="E5" s="83" t="inlineStr"/>
+      <c r="F5" s="83" t="inlineStr"/>
+      <c r="G5" s="83" t="inlineStr"/>
+      <c r="H5" s="83" t="inlineStr"/>
+      <c r="I5" s="83" t="inlineStr"/>
+      <c r="J5" s="83" t="inlineStr"/>
+      <c r="K5" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="82" t="inlineStr">
+        <is>
+          <t>D04</t>
+        </is>
+      </c>
+      <c r="B6" s="83" t="inlineStr"/>
+      <c r="C6" s="83" t="inlineStr"/>
+      <c r="D6" s="83" t="inlineStr"/>
+      <c r="E6" s="83" t="inlineStr"/>
+      <c r="F6" s="83" t="inlineStr"/>
+      <c r="G6" s="83" t="inlineStr"/>
+      <c r="H6" s="83" t="inlineStr"/>
+      <c r="I6" s="83" t="inlineStr"/>
+      <c r="J6" s="83" t="inlineStr"/>
+      <c r="K6" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="82" t="inlineStr">
+        <is>
+          <t>D05</t>
+        </is>
+      </c>
+      <c r="B7" s="83" t="inlineStr"/>
+      <c r="C7" s="83" t="inlineStr"/>
+      <c r="D7" s="83" t="inlineStr"/>
+      <c r="E7" s="83" t="inlineStr"/>
+      <c r="F7" s="83" t="inlineStr"/>
+      <c r="G7" s="83" t="inlineStr"/>
+      <c r="H7" s="83" t="inlineStr"/>
+      <c r="I7" s="83" t="inlineStr"/>
+      <c r="J7" s="83" t="inlineStr"/>
+      <c r="K7" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="82" t="inlineStr">
+        <is>
+          <t>D06</t>
+        </is>
+      </c>
+      <c r="B8" s="83" t="inlineStr"/>
+      <c r="C8" s="83" t="inlineStr"/>
+      <c r="D8" s="83" t="inlineStr"/>
+      <c r="E8" s="83" t="inlineStr"/>
+      <c r="F8" s="83" t="inlineStr"/>
+      <c r="G8" s="83" t="inlineStr"/>
+      <c r="H8" s="83" t="inlineStr"/>
+      <c r="I8" s="83" t="inlineStr"/>
+      <c r="J8" s="83" t="inlineStr"/>
+      <c r="K8" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="82" t="inlineStr">
+        <is>
+          <t>D07</t>
+        </is>
+      </c>
+      <c r="B9" s="83" t="inlineStr"/>
+      <c r="C9" s="83" t="inlineStr"/>
+      <c r="D9" s="83" t="inlineStr"/>
+      <c r="E9" s="83" t="inlineStr"/>
+      <c r="F9" s="83" t="inlineStr"/>
+      <c r="G9" s="83" t="inlineStr"/>
+      <c r="H9" s="83" t="inlineStr"/>
+      <c r="I9" s="83" t="inlineStr"/>
+      <c r="J9" s="83" t="inlineStr"/>
+      <c r="K9" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="82" t="inlineStr">
+        <is>
+          <t>D08</t>
+        </is>
+      </c>
+      <c r="B10" s="83" t="inlineStr"/>
+      <c r="C10" s="83" t="inlineStr"/>
+      <c r="D10" s="83" t="inlineStr"/>
+      <c r="E10" s="83" t="inlineStr"/>
+      <c r="F10" s="83" t="inlineStr"/>
+      <c r="G10" s="83" t="inlineStr"/>
+      <c r="H10" s="83" t="inlineStr"/>
+      <c r="I10" s="83" t="inlineStr"/>
+      <c r="J10" s="83" t="inlineStr"/>
+      <c r="K10" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="82" t="inlineStr">
+        <is>
+          <t>D09</t>
+        </is>
+      </c>
+      <c r="B11" s="83" t="inlineStr"/>
+      <c r="C11" s="83" t="inlineStr"/>
+      <c r="D11" s="83" t="inlineStr"/>
+      <c r="E11" s="83" t="inlineStr"/>
+      <c r="F11" s="83" t="inlineStr"/>
+      <c r="G11" s="83" t="inlineStr"/>
+      <c r="H11" s="83" t="inlineStr"/>
+      <c r="I11" s="83" t="inlineStr"/>
+      <c r="J11" s="83" t="inlineStr"/>
+      <c r="K11" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="82" t="inlineStr">
+        <is>
+          <t>D10</t>
+        </is>
+      </c>
+      <c r="B12" s="83" t="inlineStr"/>
+      <c r="C12" s="83" t="inlineStr"/>
+      <c r="D12" s="83" t="inlineStr"/>
+      <c r="E12" s="83" t="inlineStr"/>
+      <c r="F12" s="83" t="inlineStr"/>
+      <c r="G12" s="83" t="inlineStr"/>
+      <c r="H12" s="83" t="inlineStr"/>
+      <c r="I12" s="83" t="inlineStr"/>
+      <c r="J12" s="83" t="inlineStr"/>
+      <c r="K12" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:K1"/>
+  </mergeCells>
+  <dataValidations count="4">
+    <dataValidation sqref="D3:D12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"موظف بمرتب,بالمشوار,باليوم,من مورد نقل"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F3:F12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"شهر,مشوار,يوم,رحلة"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G3:G12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"جنيه,يورو"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K3:K12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"ناقص,اتملى,محتاج مراجعة,مش محتاجينه"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="48" customHeight="1">
+      <c r="A1" s="80" t="inlineStr">
+        <is>
+          <t>العربيات اللي بتستخدمها في التوصيل والرحلات (ملكك أو مؤجرة).</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="81" t="inlineStr">
+        <is>
+          <t>كود العربية (V01…)</t>
+        </is>
+      </c>
+      <c r="B2" s="81" t="inlineStr">
+        <is>
+          <t>الاسم / اللوحة (اختياري)</t>
+        </is>
+      </c>
+      <c r="C2" s="81" t="inlineStr">
+        <is>
+          <t>النوع</t>
+        </is>
+      </c>
+      <c r="D2" s="81" t="inlineStr">
+        <is>
+          <t>عدد الركاب</t>
+        </is>
+      </c>
+      <c r="E2" s="81" t="inlineStr">
+        <is>
+          <t>ملك ولا إيجار؟</t>
+        </is>
+      </c>
+      <c r="F2" s="81" t="inlineStr">
+        <is>
+          <t>المؤجر (لو إيجار)</t>
+        </is>
+      </c>
+      <c r="G2" s="81" t="inlineStr">
+        <is>
+          <t>سعر الإيجار</t>
+        </is>
+      </c>
+      <c r="H2" s="81" t="inlineStr">
+        <is>
+          <t>على أساس</t>
+        </is>
+      </c>
+      <c r="I2" s="81" t="inlineStr">
+        <is>
+          <t>العملة</t>
+        </is>
+      </c>
+      <c r="J2" s="81" t="inlineStr">
+        <is>
+          <t>البنزين على مين؟</t>
+        </is>
+      </c>
+      <c r="K2" s="81" t="inlineStr">
+        <is>
+          <t>ملاحظات</t>
+        </is>
+      </c>
+      <c r="L2" s="81" t="inlineStr">
+        <is>
+          <t>الحالة</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="82" t="inlineStr">
+        <is>
+          <t>V01</t>
+        </is>
+      </c>
+      <c r="B3" s="83" t="inlineStr"/>
+      <c r="C3" s="83" t="inlineStr"/>
+      <c r="D3" s="83" t="inlineStr"/>
+      <c r="E3" s="83" t="inlineStr"/>
+      <c r="F3" s="83" t="inlineStr"/>
+      <c r="G3" s="83" t="inlineStr"/>
+      <c r="H3" s="83" t="inlineStr"/>
+      <c r="I3" s="83" t="inlineStr"/>
+      <c r="J3" s="83" t="inlineStr"/>
+      <c r="K3" s="83" t="inlineStr"/>
+      <c r="L3" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="82" t="inlineStr">
+        <is>
+          <t>V02</t>
+        </is>
+      </c>
+      <c r="B4" s="83" t="inlineStr"/>
+      <c r="C4" s="83" t="inlineStr"/>
+      <c r="D4" s="83" t="inlineStr"/>
+      <c r="E4" s="83" t="inlineStr"/>
+      <c r="F4" s="83" t="inlineStr"/>
+      <c r="G4" s="83" t="inlineStr"/>
+      <c r="H4" s="83" t="inlineStr"/>
+      <c r="I4" s="83" t="inlineStr"/>
+      <c r="J4" s="83" t="inlineStr"/>
+      <c r="K4" s="83" t="inlineStr"/>
+      <c r="L4" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="82" t="inlineStr">
+        <is>
+          <t>V03</t>
+        </is>
+      </c>
+      <c r="B5" s="83" t="inlineStr"/>
+      <c r="C5" s="83" t="inlineStr"/>
+      <c r="D5" s="83" t="inlineStr"/>
+      <c r="E5" s="83" t="inlineStr"/>
+      <c r="F5" s="83" t="inlineStr"/>
+      <c r="G5" s="83" t="inlineStr"/>
+      <c r="H5" s="83" t="inlineStr"/>
+      <c r="I5" s="83" t="inlineStr"/>
+      <c r="J5" s="83" t="inlineStr"/>
+      <c r="K5" s="83" t="inlineStr"/>
+      <c r="L5" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="82" t="inlineStr">
+        <is>
+          <t>V04</t>
+        </is>
+      </c>
+      <c r="B6" s="83" t="inlineStr"/>
+      <c r="C6" s="83" t="inlineStr"/>
+      <c r="D6" s="83" t="inlineStr"/>
+      <c r="E6" s="83" t="inlineStr"/>
+      <c r="F6" s="83" t="inlineStr"/>
+      <c r="G6" s="83" t="inlineStr"/>
+      <c r="H6" s="83" t="inlineStr"/>
+      <c r="I6" s="83" t="inlineStr"/>
+      <c r="J6" s="83" t="inlineStr"/>
+      <c r="K6" s="83" t="inlineStr"/>
+      <c r="L6" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="82" t="inlineStr">
+        <is>
+          <t>V05</t>
+        </is>
+      </c>
+      <c r="B7" s="83" t="inlineStr"/>
+      <c r="C7" s="83" t="inlineStr"/>
+      <c r="D7" s="83" t="inlineStr"/>
+      <c r="E7" s="83" t="inlineStr"/>
+      <c r="F7" s="83" t="inlineStr"/>
+      <c r="G7" s="83" t="inlineStr"/>
+      <c r="H7" s="83" t="inlineStr"/>
+      <c r="I7" s="83" t="inlineStr"/>
+      <c r="J7" s="83" t="inlineStr"/>
+      <c r="K7" s="83" t="inlineStr"/>
+      <c r="L7" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="82" t="inlineStr">
+        <is>
+          <t>V06</t>
+        </is>
+      </c>
+      <c r="B8" s="83" t="inlineStr"/>
+      <c r="C8" s="83" t="inlineStr"/>
+      <c r="D8" s="83" t="inlineStr"/>
+      <c r="E8" s="83" t="inlineStr"/>
+      <c r="F8" s="83" t="inlineStr"/>
+      <c r="G8" s="83" t="inlineStr"/>
+      <c r="H8" s="83" t="inlineStr"/>
+      <c r="I8" s="83" t="inlineStr"/>
+      <c r="J8" s="83" t="inlineStr"/>
+      <c r="K8" s="83" t="inlineStr"/>
+      <c r="L8" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="82" t="inlineStr">
+        <is>
+          <t>V07</t>
+        </is>
+      </c>
+      <c r="B9" s="83" t="inlineStr"/>
+      <c r="C9" s="83" t="inlineStr"/>
+      <c r="D9" s="83" t="inlineStr"/>
+      <c r="E9" s="83" t="inlineStr"/>
+      <c r="F9" s="83" t="inlineStr"/>
+      <c r="G9" s="83" t="inlineStr"/>
+      <c r="H9" s="83" t="inlineStr"/>
+      <c r="I9" s="83" t="inlineStr"/>
+      <c r="J9" s="83" t="inlineStr"/>
+      <c r="K9" s="83" t="inlineStr"/>
+      <c r="L9" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="82" t="inlineStr">
+        <is>
+          <t>V08</t>
+        </is>
+      </c>
+      <c r="B10" s="83" t="inlineStr"/>
+      <c r="C10" s="83" t="inlineStr"/>
+      <c r="D10" s="83" t="inlineStr"/>
+      <c r="E10" s="83" t="inlineStr"/>
+      <c r="F10" s="83" t="inlineStr"/>
+      <c r="G10" s="83" t="inlineStr"/>
+      <c r="H10" s="83" t="inlineStr"/>
+      <c r="I10" s="83" t="inlineStr"/>
+      <c r="J10" s="83" t="inlineStr"/>
+      <c r="K10" s="83" t="inlineStr"/>
+      <c r="L10" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="82" t="inlineStr">
+        <is>
+          <t>V09</t>
+        </is>
+      </c>
+      <c r="B11" s="83" t="inlineStr"/>
+      <c r="C11" s="83" t="inlineStr"/>
+      <c r="D11" s="83" t="inlineStr"/>
+      <c r="E11" s="83" t="inlineStr"/>
+      <c r="F11" s="83" t="inlineStr"/>
+      <c r="G11" s="83" t="inlineStr"/>
+      <c r="H11" s="83" t="inlineStr"/>
+      <c r="I11" s="83" t="inlineStr"/>
+      <c r="J11" s="83" t="inlineStr"/>
+      <c r="K11" s="83" t="inlineStr"/>
+      <c r="L11" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="82" t="inlineStr">
+        <is>
+          <t>V10</t>
+        </is>
+      </c>
+      <c r="B12" s="83" t="inlineStr"/>
+      <c r="C12" s="83" t="inlineStr"/>
+      <c r="D12" s="83" t="inlineStr"/>
+      <c r="E12" s="83" t="inlineStr"/>
+      <c r="F12" s="83" t="inlineStr"/>
+      <c r="G12" s="83" t="inlineStr"/>
+      <c r="H12" s="83" t="inlineStr"/>
+      <c r="I12" s="83" t="inlineStr"/>
+      <c r="J12" s="83" t="inlineStr"/>
+      <c r="K12" s="83" t="inlineStr"/>
+      <c r="L12" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:L1"/>
+  </mergeCells>
+  <dataValidations count="6">
+    <dataValidation sqref="C3:C12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"سيدان,SUV,هايس / ميني باص,كوستر,أتوبيس,جيب,أخرى"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E3:E12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"ملك,إيجار"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H3:H12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"مشوار,يوم,شهر"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I3:I12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"جنيه,يورو"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J3:J12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"علينا,على المؤجر,على السواق"</formula1>
+    </dataValidation>
+    <dataValidation sqref="L3:L12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"ناقص,اتملى,محتاج مراجعة,مش محتاجينه"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -6990,6 +8918,748 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="48" customHeight="1">
+      <c r="A1" s="80" t="inlineStr">
+        <is>
+          <t>قواعد الحساب مع الموردين والسواقين والعمولات. اكتب ردّك في العمود الأصفر.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="81" t="inlineStr">
+        <is>
+          <t>الكود (key)</t>
+        </is>
+      </c>
+      <c r="B2" s="81" t="inlineStr">
+        <is>
+          <t>السؤال</t>
+        </is>
+      </c>
+      <c r="C2" s="81" t="inlineStr">
+        <is>
+          <t>ردّك</t>
+        </is>
+      </c>
+      <c r="D2" s="81" t="inlineStr">
+        <is>
+          <t>مثال</t>
+        </is>
+      </c>
+      <c r="E2" s="81" t="inlineStr">
+        <is>
+          <t>الحالة</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="82" t="inlineStr">
+        <is>
+          <t>settle_approver</t>
+        </is>
+      </c>
+      <c r="B3" s="82" t="inlineStr">
+        <is>
+          <t>مين يعتمد الدفع للمورد أو السواق؟</t>
+        </is>
+      </c>
+      <c r="C3" s="83" t="inlineStr"/>
+      <c r="D3" s="82" t="inlineStr">
+        <is>
+          <t>محمد بس / محمد أو المدير</t>
+        </is>
+      </c>
+      <c r="E3" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="82" t="inlineStr">
+        <is>
+          <t>settle_limit</t>
+        </is>
+      </c>
+      <c r="B4" s="82" t="inlineStr">
+        <is>
+          <t>فيه مبلغ يقدر المدير يدفعه من غير اعتمادك؟ كام؟</t>
+        </is>
+      </c>
+      <c r="C4" s="83" t="inlineStr"/>
+      <c r="D4" s="82" t="inlineStr">
+        <is>
+          <t>لحد 5000 جنيه</t>
+        </is>
+      </c>
+      <c r="E4" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="82" t="inlineStr">
+        <is>
+          <t>settle_fx</t>
+        </is>
+      </c>
+      <c r="B5" s="82" t="inlineStr">
+        <is>
+          <t>الحساب مع الموردين بالجنيه بيتحسب بنفس سعر اليوم اللي المدير بيحدده؟</t>
+        </is>
+      </c>
+      <c r="C5" s="83" t="inlineStr"/>
+      <c r="D5" s="82" t="inlineStr">
+        <is>
+          <t>آه / لأ، بسعر متفق عليه</t>
+        </is>
+      </c>
+      <c r="E5" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="82" t="inlineStr">
+        <is>
+          <t>commission_sales</t>
+        </is>
+      </c>
+      <c r="B6" s="82" t="inlineStr">
+        <is>
+          <t>فيه عمولة لموظف المبيعات؟ كام ولمين؟</t>
+        </is>
+      </c>
+      <c r="C6" s="83" t="inlineStr"/>
+      <c r="D6" s="82" t="inlineStr">
+        <is>
+          <t>5% من البيع للي جاب العميل</t>
+        </is>
+      </c>
+      <c r="E6" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="82" t="inlineStr">
+        <is>
+          <t>commission_hotel</t>
+        </is>
+      </c>
+      <c r="B7" s="82" t="inlineStr">
+        <is>
+          <t>فيه عمولة لفندق أو ريسبشن بيجيب عملاء؟ كام؟</t>
+        </is>
+      </c>
+      <c r="C7" s="83" t="inlineStr"/>
+      <c r="D7" s="82" t="inlineStr">
+        <is>
+          <t>10 يورو للفرد / 10%</t>
+        </is>
+      </c>
+      <c r="E7" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="82" t="inlineStr">
+        <is>
+          <t>commission_paid_when</t>
+        </is>
+      </c>
+      <c r="B8" s="82" t="inlineStr">
+        <is>
+          <t>العمولات بتتدفع إمتى وإزاي؟</t>
+        </is>
+      </c>
+      <c r="C8" s="83" t="inlineStr"/>
+      <c r="D8" s="82" t="inlineStr">
+        <is>
+          <t>آخر الشهر كاش</t>
+        </is>
+      </c>
+      <c r="E8" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="82" t="inlineStr">
+        <is>
+          <t>refund_rule</t>
+        </is>
+      </c>
+      <c r="B9" s="82" t="inlineStr">
+        <is>
+          <t>لو حجز مدفوع اتلغى، الفلوس بترجع للعميل إزاي ومين يعتمد؟</t>
+        </is>
+      </c>
+      <c r="C9" s="83" t="inlineStr"/>
+      <c r="D9" s="82" t="inlineStr">
+        <is>
+          <t>كاش من المكتب بعد اعتماد محمد</t>
+        </is>
+      </c>
+      <c r="E9" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="82" t="inlineStr">
+        <is>
+          <t>cash_box</t>
+        </is>
+      </c>
+      <c r="B10" s="82" t="inlineStr">
+        <is>
+          <t>فيه خزنة/درج كاش في المكتب بيتقفل آخر اليوم؟ مين مسؤول عنه؟</t>
+        </is>
+      </c>
+      <c r="C10" s="83" t="inlineStr"/>
+      <c r="D10" s="82" t="inlineStr">
+        <is>
+          <t>موظف الاستقبال + تسليم يومي</t>
+        </is>
+      </c>
+      <c r="E10" s="82" t="inlineStr">
+        <is>
+          <t>ناقص</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="E3:E10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"ناقص,اتملى,محتاج مراجعة,مش محتاجينه"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="48" customHeight="1">
+      <c r="A1" s="80" t="inlineStr">
+        <is>
+          <t>المصاريف اللي بتدفعها انت على كل رحلة غير المورد (رسوم دخول، مرشد، أكل، مية…). سيب الخانة فاضية لو مش موجودة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="81" t="inlineStr">
+        <is>
+          <t>كود الرحلة</t>
+        </is>
+      </c>
+      <c r="B2" s="81" t="inlineStr">
+        <is>
+          <t>رسوم دخول (للفرد)</t>
+        </is>
+      </c>
+      <c r="C2" s="81" t="inlineStr">
+        <is>
+          <t>مرشد (للرحلة)</t>
+        </is>
+      </c>
+      <c r="D2" s="81" t="inlineStr">
+        <is>
+          <t>أكل (للفرد)</t>
+        </is>
+      </c>
+      <c r="E2" s="81" t="inlineStr">
+        <is>
+          <t>مية/مشروبات (للفرد)</t>
+        </is>
+      </c>
+      <c r="F2" s="81" t="inlineStr">
+        <is>
+          <t>تكاليف تانية</t>
+        </is>
+      </c>
+      <c r="G2" s="81" t="inlineStr">
+        <is>
+          <t>العملة</t>
+        </is>
+      </c>
+      <c r="H2" s="81" t="inlineStr">
+        <is>
+          <t>مين بيدفعها؟</t>
+        </is>
+      </c>
+      <c r="I2" s="81" t="inlineStr">
+        <is>
+          <t>ملاحظات</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="82" t="inlineStr">
+        <is>
+          <t>super-safari-adventure</t>
+        </is>
+      </c>
+      <c r="B3" s="83" t="inlineStr"/>
+      <c r="C3" s="83" t="inlineStr"/>
+      <c r="D3" s="83" t="inlineStr"/>
+      <c r="E3" s="83" t="inlineStr"/>
+      <c r="F3" s="83" t="inlineStr"/>
+      <c r="G3" s="83" t="inlineStr"/>
+      <c r="H3" s="83" t="inlineStr"/>
+      <c r="I3" s="83" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="82" t="inlineStr">
+        <is>
+          <t>sunset-quad-bike</t>
+        </is>
+      </c>
+      <c r="B4" s="83" t="inlineStr"/>
+      <c r="C4" s="83" t="inlineStr"/>
+      <c r="D4" s="83" t="inlineStr"/>
+      <c r="E4" s="83" t="inlineStr"/>
+      <c r="F4" s="83" t="inlineStr"/>
+      <c r="G4" s="83" t="inlineStr"/>
+      <c r="H4" s="83" t="inlineStr"/>
+      <c r="I4" s="83" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="82" t="inlineStr">
+        <is>
+          <t>double-buggy-camel-ride</t>
+        </is>
+      </c>
+      <c r="B5" s="83" t="inlineStr"/>
+      <c r="C5" s="83" t="inlineStr"/>
+      <c r="D5" s="83" t="inlineStr"/>
+      <c r="E5" s="83" t="inlineStr"/>
+      <c r="F5" s="83" t="inlineStr"/>
+      <c r="G5" s="83" t="inlineStr"/>
+      <c r="H5" s="83" t="inlineStr"/>
+      <c r="I5" s="83" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="82" t="inlineStr">
+        <is>
+          <t>bedouin-dinner-camel-ride</t>
+        </is>
+      </c>
+      <c r="B6" s="83" t="inlineStr"/>
+      <c r="C6" s="83" t="inlineStr"/>
+      <c r="D6" s="83" t="inlineStr"/>
+      <c r="E6" s="83" t="inlineStr"/>
+      <c r="F6" s="83" t="inlineStr"/>
+      <c r="G6" s="83" t="inlineStr"/>
+      <c r="H6" s="83" t="inlineStr"/>
+      <c r="I6" s="83" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="82" t="inlineStr">
+        <is>
+          <t>dahab-colored-canyon</t>
+        </is>
+      </c>
+      <c r="B7" s="83" t="inlineStr"/>
+      <c r="C7" s="83" t="inlineStr"/>
+      <c r="D7" s="83" t="inlineStr"/>
+      <c r="E7" s="83" t="inlineStr"/>
+      <c r="F7" s="83" t="inlineStr"/>
+      <c r="G7" s="83" t="inlineStr"/>
+      <c r="H7" s="83" t="inlineStr"/>
+      <c r="I7" s="83" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="82" t="inlineStr">
+        <is>
+          <t>camel-horse-ride</t>
+        </is>
+      </c>
+      <c r="B8" s="83" t="inlineStr"/>
+      <c r="C8" s="83" t="inlineStr"/>
+      <c r="D8" s="83" t="inlineStr"/>
+      <c r="E8" s="83" t="inlineStr"/>
+      <c r="F8" s="83" t="inlineStr"/>
+      <c r="G8" s="83" t="inlineStr"/>
+      <c r="H8" s="83" t="inlineStr"/>
+      <c r="I8" s="83" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="82" t="inlineStr">
+        <is>
+          <t>ras-mohamed-white-island-boat</t>
+        </is>
+      </c>
+      <c r="B9" s="83" t="inlineStr"/>
+      <c r="C9" s="83" t="inlineStr"/>
+      <c r="D9" s="83" t="inlineStr"/>
+      <c r="E9" s="83" t="inlineStr"/>
+      <c r="F9" s="83" t="inlineStr"/>
+      <c r="G9" s="83" t="inlineStr"/>
+      <c r="H9" s="83" t="inlineStr"/>
+      <c r="I9" s="83" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="82" t="inlineStr">
+        <is>
+          <t>evening-cruise</t>
+        </is>
+      </c>
+      <c r="B10" s="83" t="inlineStr"/>
+      <c r="C10" s="83" t="inlineStr"/>
+      <c r="D10" s="83" t="inlineStr"/>
+      <c r="E10" s="83" t="inlineStr"/>
+      <c r="F10" s="83" t="inlineStr"/>
+      <c r="G10" s="83" t="inlineStr"/>
+      <c r="H10" s="83" t="inlineStr"/>
+      <c r="I10" s="83" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="82" t="inlineStr">
+        <is>
+          <t>glass-bottom-boat</t>
+        </is>
+      </c>
+      <c r="B11" s="83" t="inlineStr"/>
+      <c r="C11" s="83" t="inlineStr"/>
+      <c r="D11" s="83" t="inlineStr"/>
+      <c r="E11" s="83" t="inlineStr"/>
+      <c r="F11" s="83" t="inlineStr"/>
+      <c r="G11" s="83" t="inlineStr"/>
+      <c r="H11" s="83" t="inlineStr"/>
+      <c r="I11" s="83" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="82" t="inlineStr">
+        <is>
+          <t>diving-course</t>
+        </is>
+      </c>
+      <c r="B12" s="83" t="inlineStr"/>
+      <c r="C12" s="83" t="inlineStr"/>
+      <c r="D12" s="83" t="inlineStr"/>
+      <c r="E12" s="83" t="inlineStr"/>
+      <c r="F12" s="83" t="inlineStr"/>
+      <c r="G12" s="83" t="inlineStr"/>
+      <c r="H12" s="83" t="inlineStr"/>
+      <c r="I12" s="83" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="82" t="inlineStr">
+        <is>
+          <t>sinai-dream-sailboat</t>
+        </is>
+      </c>
+      <c r="B13" s="83" t="inlineStr"/>
+      <c r="C13" s="83" t="inlineStr"/>
+      <c r="D13" s="83" t="inlineStr"/>
+      <c r="E13" s="83" t="inlineStr"/>
+      <c r="F13" s="83" t="inlineStr"/>
+      <c r="G13" s="83" t="inlineStr"/>
+      <c r="H13" s="83" t="inlineStr"/>
+      <c r="I13" s="83" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="82" t="inlineStr">
+        <is>
+          <t>ras-mohamed-by-bus</t>
+        </is>
+      </c>
+      <c r="B14" s="83" t="inlineStr"/>
+      <c r="C14" s="83" t="inlineStr"/>
+      <c r="D14" s="83" t="inlineStr"/>
+      <c r="E14" s="83" t="inlineStr"/>
+      <c r="F14" s="83" t="inlineStr"/>
+      <c r="G14" s="83" t="inlineStr"/>
+      <c r="H14" s="83" t="inlineStr"/>
+      <c r="I14" s="83" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="82" t="inlineStr">
+        <is>
+          <t>banana-boat</t>
+        </is>
+      </c>
+      <c r="B15" s="83" t="inlineStr"/>
+      <c r="C15" s="83" t="inlineStr"/>
+      <c r="D15" s="83" t="inlineStr"/>
+      <c r="E15" s="83" t="inlineStr"/>
+      <c r="F15" s="83" t="inlineStr"/>
+      <c r="G15" s="83" t="inlineStr"/>
+      <c r="H15" s="83" t="inlineStr"/>
+      <c r="I15" s="83" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="82" t="inlineStr">
+        <is>
+          <t>parasailing-adventure</t>
+        </is>
+      </c>
+      <c r="B16" s="83" t="inlineStr"/>
+      <c r="C16" s="83" t="inlineStr"/>
+      <c r="D16" s="83" t="inlineStr"/>
+      <c r="E16" s="83" t="inlineStr"/>
+      <c r="F16" s="83" t="inlineStr"/>
+      <c r="G16" s="83" t="inlineStr"/>
+      <c r="H16" s="83" t="inlineStr"/>
+      <c r="I16" s="83" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="82" t="inlineStr">
+        <is>
+          <t>speed-boat-adventure</t>
+        </is>
+      </c>
+      <c r="B17" s="83" t="inlineStr"/>
+      <c r="C17" s="83" t="inlineStr"/>
+      <c r="D17" s="83" t="inlineStr"/>
+      <c r="E17" s="83" t="inlineStr"/>
+      <c r="F17" s="83" t="inlineStr"/>
+      <c r="G17" s="83" t="inlineStr"/>
+      <c r="H17" s="83" t="inlineStr"/>
+      <c r="I17" s="83" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="82" t="inlineStr">
+        <is>
+          <t>submarine</t>
+        </is>
+      </c>
+      <c r="B18" s="83" t="inlineStr"/>
+      <c r="C18" s="83" t="inlineStr"/>
+      <c r="D18" s="83" t="inlineStr"/>
+      <c r="E18" s="83" t="inlineStr"/>
+      <c r="F18" s="83" t="inlineStr"/>
+      <c r="G18" s="83" t="inlineStr"/>
+      <c r="H18" s="83" t="inlineStr"/>
+      <c r="I18" s="83" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="82" t="inlineStr">
+        <is>
+          <t>tiran-island-boat-trip</t>
+        </is>
+      </c>
+      <c r="B19" s="83" t="inlineStr"/>
+      <c r="C19" s="83" t="inlineStr"/>
+      <c r="D19" s="83" t="inlineStr"/>
+      <c r="E19" s="83" t="inlineStr"/>
+      <c r="F19" s="83" t="inlineStr"/>
+      <c r="G19" s="83" t="inlineStr"/>
+      <c r="H19" s="83" t="inlineStr"/>
+      <c r="I19" s="83" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="82" t="inlineStr">
+        <is>
+          <t>tube-boat</t>
+        </is>
+      </c>
+      <c r="B20" s="83" t="inlineStr"/>
+      <c r="C20" s="83" t="inlineStr"/>
+      <c r="D20" s="83" t="inlineStr"/>
+      <c r="E20" s="83" t="inlineStr"/>
+      <c r="F20" s="83" t="inlineStr"/>
+      <c r="G20" s="83" t="inlineStr"/>
+      <c r="H20" s="83" t="inlineStr"/>
+      <c r="I20" s="83" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="82" t="inlineStr">
+        <is>
+          <t>cairo-by-bus</t>
+        </is>
+      </c>
+      <c r="B21" s="83" t="inlineStr"/>
+      <c r="C21" s="83" t="inlineStr"/>
+      <c r="D21" s="83" t="inlineStr"/>
+      <c r="E21" s="83" t="inlineStr"/>
+      <c r="F21" s="83" t="inlineStr"/>
+      <c r="G21" s="83" t="inlineStr"/>
+      <c r="H21" s="83" t="inlineStr"/>
+      <c r="I21" s="83" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="82" t="inlineStr">
+        <is>
+          <t>cairo-by-plane</t>
+        </is>
+      </c>
+      <c r="B22" s="83" t="inlineStr"/>
+      <c r="C22" s="83" t="inlineStr"/>
+      <c r="D22" s="83" t="inlineStr"/>
+      <c r="E22" s="83" t="inlineStr"/>
+      <c r="F22" s="83" t="inlineStr"/>
+      <c r="G22" s="83" t="inlineStr"/>
+      <c r="H22" s="83" t="inlineStr"/>
+      <c r="I22" s="83" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="82" t="inlineStr">
+        <is>
+          <t>mount-sinai-st-catherine</t>
+        </is>
+      </c>
+      <c r="B23" s="83" t="inlineStr"/>
+      <c r="C23" s="83" t="inlineStr"/>
+      <c r="D23" s="83" t="inlineStr"/>
+      <c r="E23" s="83" t="inlineStr"/>
+      <c r="F23" s="83" t="inlineStr"/>
+      <c r="G23" s="83" t="inlineStr"/>
+      <c r="H23" s="83" t="inlineStr"/>
+      <c r="I23" s="83" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="82" t="inlineStr">
+        <is>
+          <t>luxor-by-plane</t>
+        </is>
+      </c>
+      <c r="B24" s="83" t="inlineStr"/>
+      <c r="C24" s="83" t="inlineStr"/>
+      <c r="D24" s="83" t="inlineStr"/>
+      <c r="E24" s="83" t="inlineStr"/>
+      <c r="F24" s="83" t="inlineStr"/>
+      <c r="G24" s="83" t="inlineStr"/>
+      <c r="H24" s="83" t="inlineStr"/>
+      <c r="I24" s="83" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="82" t="inlineStr">
+        <is>
+          <t>st-catherine-dahab</t>
+        </is>
+      </c>
+      <c r="B25" s="83" t="inlineStr"/>
+      <c r="C25" s="83" t="inlineStr"/>
+      <c r="D25" s="83" t="inlineStr"/>
+      <c r="E25" s="83" t="inlineStr"/>
+      <c r="F25" s="83" t="inlineStr"/>
+      <c r="G25" s="83" t="inlineStr"/>
+      <c r="H25" s="83" t="inlineStr"/>
+      <c r="I25" s="83" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="82" t="inlineStr">
+        <is>
+          <t>turkish-bath</t>
+        </is>
+      </c>
+      <c r="B26" s="83" t="inlineStr"/>
+      <c r="C26" s="83" t="inlineStr"/>
+      <c r="D26" s="83" t="inlineStr"/>
+      <c r="E26" s="83" t="inlineStr"/>
+      <c r="F26" s="83" t="inlineStr"/>
+      <c r="G26" s="83" t="inlineStr"/>
+      <c r="H26" s="83" t="inlineStr"/>
+      <c r="I26" s="83" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="82" t="inlineStr">
+        <is>
+          <t>dolphin-show</t>
+        </is>
+      </c>
+      <c r="B27" s="83" t="inlineStr"/>
+      <c r="C27" s="83" t="inlineStr"/>
+      <c r="D27" s="83" t="inlineStr"/>
+      <c r="E27" s="83" t="inlineStr"/>
+      <c r="F27" s="83" t="inlineStr"/>
+      <c r="G27" s="83" t="inlineStr"/>
+      <c r="H27" s="83" t="inlineStr"/>
+      <c r="I27" s="83" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="82" t="inlineStr">
+        <is>
+          <t>swimming-with-dolphins</t>
+        </is>
+      </c>
+      <c r="B28" s="83" t="inlineStr"/>
+      <c r="C28" s="83" t="inlineStr"/>
+      <c r="D28" s="83" t="inlineStr"/>
+      <c r="E28" s="83" t="inlineStr"/>
+      <c r="F28" s="83" t="inlineStr"/>
+      <c r="G28" s="83" t="inlineStr"/>
+      <c r="H28" s="83" t="inlineStr"/>
+      <c r="I28" s="83" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="82" t="inlineStr">
+        <is>
+          <t>sharm-airport-transfer</t>
+        </is>
+      </c>
+      <c r="B29" s="83" t="inlineStr"/>
+      <c r="C29" s="83" t="inlineStr"/>
+      <c r="D29" s="83" t="inlineStr"/>
+      <c r="E29" s="83" t="inlineStr"/>
+      <c r="F29" s="83" t="inlineStr"/>
+      <c r="G29" s="83" t="inlineStr"/>
+      <c r="H29" s="83" t="inlineStr"/>
+      <c r="I29" s="83" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:I1"/>
+  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="G3:G29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"جنيه,يورو"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H3:H29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"احنا,المورد,العميل"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
docs(safari-owner-data): merge owner's supplier, driver, cost and company answers (2026-10-06)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/clients/safari-tours-sharm/owner-data/safari-tours-owner-data-hub.xlsx
+++ b/clients/safari-tours-sharm/owner-data/safari-tours-owner-data-hub.xlsx
@@ -31,7 +31,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+  </numFmts>
   <fonts count="17">
     <font>
       <name val="Calibri"/>
@@ -243,7 +245,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="84">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -462,6 +464,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1559,7 +1564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1734,6 +1739,23 @@
       <c r="C10" t="inlineStr">
         <is>
           <t>أضاف شيتات الموردين وأسعار الموردين والسواقين والعربيات والتكاليف والتسويات وتكاليف الرحلات — بطلب محمد «اعملها».</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>محمد (عن طريق Claude)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>دمج ملف محمد «safari-tours-owner-data (1).xlsx»: 5 موردين، أسعار الموردين لكل الرحلات، 4 سواقين، تكاليف الرحلات، وبيانات الشركة (ساعات الدعم 24 ساعة، اللغات، سنة البداية، مفيش ترخيص سياحة حاليًا). العربيات فاضية لحد ما تتوفر البيانات.</t>
         </is>
       </c>
     </row>
@@ -6441,18 +6463,58 @@
           <t>S01</t>
         </is>
       </c>
-      <c r="B3" s="83" t="inlineStr"/>
-      <c r="C3" s="83" t="inlineStr"/>
+      <c r="B3" s="83" t="inlineStr">
+        <is>
+          <t>حامد السندباد</t>
+        </is>
+      </c>
+      <c r="C3" s="83" t="inlineStr">
+        <is>
+          <t>غوص/سنوركل</t>
+        </is>
+      </c>
       <c r="D3" s="83" t="inlineStr"/>
-      <c r="E3" s="83" t="inlineStr"/>
-      <c r="F3" s="83" t="inlineStr"/>
-      <c r="G3" s="83" t="inlineStr"/>
-      <c r="H3" s="83" t="inlineStr"/>
-      <c r="I3" s="83" t="inlineStr"/>
-      <c r="J3" s="83" t="inlineStr"/>
-      <c r="K3" s="83" t="inlineStr"/>
-      <c r="L3" s="83" t="inlineStr"/>
-      <c r="M3" s="83" t="inlineStr"/>
+      <c r="E3" s="83" t="inlineStr">
+        <is>
+          <t>حامد</t>
+        </is>
+      </c>
+      <c r="F3" s="83" t="n">
+        <v>1015048400</v>
+      </c>
+      <c r="G3" s="83" t="inlineStr">
+        <is>
+          <t>واتساب</t>
+        </is>
+      </c>
+      <c r="H3" s="83" t="n">
+        <v>24</v>
+      </c>
+      <c r="I3" s="83" t="inlineStr">
+        <is>
+          <t>لكل فرد</t>
+        </is>
+      </c>
+      <c r="J3" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
+      <c r="K3" s="83" t="inlineStr">
+        <is>
+          <t>بعد كل رحلة</t>
+        </is>
+      </c>
+      <c r="L3" s="83" t="inlineStr">
+        <is>
+          <t>إنستاباي</t>
+        </is>
+      </c>
+      <c r="M3" s="83" t="inlineStr">
+        <is>
+          <t>خصم</t>
+        </is>
+      </c>
       <c r="N3" s="83" t="inlineStr"/>
       <c r="O3" s="82" t="inlineStr">
         <is>
@@ -6466,18 +6528,50 @@
           <t>S02</t>
         </is>
       </c>
-      <c r="B4" s="83" t="inlineStr"/>
-      <c r="C4" s="83" t="inlineStr"/>
+      <c r="B4" s="83" t="inlineStr">
+        <is>
+          <t>محمد بنوراما نعمه</t>
+        </is>
+      </c>
+      <c r="C4" s="83" t="inlineStr">
+        <is>
+          <t>كواد/باجي/سفاري</t>
+        </is>
+      </c>
       <c r="D4" s="83" t="inlineStr"/>
       <c r="E4" s="83" t="inlineStr"/>
-      <c r="F4" s="83" t="inlineStr"/>
-      <c r="G4" s="83" t="inlineStr"/>
-      <c r="H4" s="83" t="inlineStr"/>
-      <c r="I4" s="83" t="inlineStr"/>
-      <c r="J4" s="83" t="inlineStr"/>
+      <c r="F4" s="83" t="n">
+        <v>1156405032</v>
+      </c>
+      <c r="G4" s="83" t="inlineStr">
+        <is>
+          <t>واتساب</t>
+        </is>
+      </c>
+      <c r="H4" s="83" t="n">
+        <v>24</v>
+      </c>
+      <c r="I4" s="83" t="inlineStr">
+        <is>
+          <t>لكل فرد</t>
+        </is>
+      </c>
+      <c r="J4" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
       <c r="K4" s="83" t="inlineStr"/>
-      <c r="L4" s="83" t="inlineStr"/>
-      <c r="M4" s="83" t="inlineStr"/>
+      <c r="L4" s="83" t="inlineStr">
+        <is>
+          <t>محفظة إلكترونية</t>
+        </is>
+      </c>
+      <c r="M4" s="83" t="inlineStr">
+        <is>
+          <t>خصم</t>
+        </is>
+      </c>
       <c r="N4" s="83" t="inlineStr"/>
       <c r="O4" s="82" t="inlineStr">
         <is>
@@ -6491,18 +6585,58 @@
           <t>S03</t>
         </is>
       </c>
-      <c r="B5" s="83" t="inlineStr"/>
-      <c r="C5" s="83" t="inlineStr"/>
+      <c r="B5" s="83" t="inlineStr">
+        <is>
+          <t>فيري ترافل</t>
+        </is>
+      </c>
+      <c r="C5" s="83" t="inlineStr">
+        <is>
+          <t>كواد/باجي/سفاري</t>
+        </is>
+      </c>
       <c r="D5" s="83" t="inlineStr"/>
-      <c r="E5" s="83" t="inlineStr"/>
-      <c r="F5" s="83" t="inlineStr"/>
-      <c r="G5" s="83" t="inlineStr"/>
-      <c r="H5" s="83" t="inlineStr"/>
-      <c r="I5" s="83" t="inlineStr"/>
-      <c r="J5" s="83" t="inlineStr"/>
-      <c r="K5" s="83" t="inlineStr"/>
-      <c r="L5" s="83" t="inlineStr"/>
-      <c r="M5" s="83" t="inlineStr"/>
+      <c r="E5" s="83" t="inlineStr">
+        <is>
+          <t>هيثم</t>
+        </is>
+      </c>
+      <c r="F5" s="83" t="n">
+        <v>1002237211</v>
+      </c>
+      <c r="G5" s="83" t="inlineStr">
+        <is>
+          <t>واتساب</t>
+        </is>
+      </c>
+      <c r="H5" s="83" t="n">
+        <v>24</v>
+      </c>
+      <c r="I5" s="83" t="inlineStr">
+        <is>
+          <t>لكل فرد</t>
+        </is>
+      </c>
+      <c r="J5" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
+      <c r="K5" s="83" t="inlineStr">
+        <is>
+          <t>بعد كل رحلة</t>
+        </is>
+      </c>
+      <c r="L5" s="83" t="inlineStr">
+        <is>
+          <t>كاش</t>
+        </is>
+      </c>
+      <c r="M5" s="83" t="inlineStr">
+        <is>
+          <t>خصم</t>
+        </is>
+      </c>
       <c r="N5" s="83" t="inlineStr"/>
       <c r="O5" s="82" t="inlineStr">
         <is>
@@ -6516,18 +6650,58 @@
           <t>S04</t>
         </is>
       </c>
-      <c r="B6" s="83" t="inlineStr"/>
-      <c r="C6" s="83" t="inlineStr"/>
+      <c r="B6" s="83" t="inlineStr">
+        <is>
+          <t>عبد الرحمن دلتا</t>
+        </is>
+      </c>
+      <c r="C6" s="83" t="inlineStr">
+        <is>
+          <t>غوص/سنوركل</t>
+        </is>
+      </c>
       <c r="D6" s="83" t="inlineStr"/>
-      <c r="E6" s="83" t="inlineStr"/>
-      <c r="F6" s="83" t="inlineStr"/>
-      <c r="G6" s="83" t="inlineStr"/>
-      <c r="H6" s="83" t="inlineStr"/>
-      <c r="I6" s="83" t="inlineStr"/>
-      <c r="J6" s="83" t="inlineStr"/>
-      <c r="K6" s="83" t="inlineStr"/>
-      <c r="L6" s="83" t="inlineStr"/>
-      <c r="M6" s="83" t="inlineStr"/>
+      <c r="E6" s="83" t="inlineStr">
+        <is>
+          <t>عبده</t>
+        </is>
+      </c>
+      <c r="F6" s="83" t="n">
+        <v>1025965216</v>
+      </c>
+      <c r="G6" s="83" t="inlineStr">
+        <is>
+          <t>تليفون</t>
+        </is>
+      </c>
+      <c r="H6" s="83" t="n">
+        <v>24</v>
+      </c>
+      <c r="I6" s="83" t="inlineStr">
+        <is>
+          <t>لكل فرد</t>
+        </is>
+      </c>
+      <c r="J6" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
+      <c r="K6" s="83" t="inlineStr">
+        <is>
+          <t>بعد كل رحلة</t>
+        </is>
+      </c>
+      <c r="L6" s="83" t="inlineStr">
+        <is>
+          <t>كاش</t>
+        </is>
+      </c>
+      <c r="M6" s="83" t="inlineStr">
+        <is>
+          <t>خصم</t>
+        </is>
+      </c>
       <c r="N6" s="83" t="inlineStr"/>
       <c r="O6" s="82" t="inlineStr">
         <is>
@@ -6541,18 +6715,58 @@
           <t>S05</t>
         </is>
       </c>
-      <c r="B7" s="83" t="inlineStr"/>
-      <c r="C7" s="83" t="inlineStr"/>
+      <c r="B7" s="83" t="inlineStr">
+        <is>
+          <t>معتز انمشين</t>
+        </is>
+      </c>
+      <c r="C7" s="83" t="inlineStr">
+        <is>
+          <t>كواد/باجي/سفاري</t>
+        </is>
+      </c>
       <c r="D7" s="83" t="inlineStr"/>
-      <c r="E7" s="83" t="inlineStr"/>
-      <c r="F7" s="83" t="inlineStr"/>
-      <c r="G7" s="83" t="inlineStr"/>
-      <c r="H7" s="83" t="inlineStr"/>
-      <c r="I7" s="83" t="inlineStr"/>
-      <c r="J7" s="83" t="inlineStr"/>
-      <c r="K7" s="83" t="inlineStr"/>
-      <c r="L7" s="83" t="inlineStr"/>
-      <c r="M7" s="83" t="inlineStr"/>
+      <c r="E7" s="83" t="inlineStr">
+        <is>
+          <t>معتز</t>
+        </is>
+      </c>
+      <c r="F7" s="83" t="n">
+        <v>1116211823</v>
+      </c>
+      <c r="G7" s="83" t="inlineStr">
+        <is>
+          <t>تليفون</t>
+        </is>
+      </c>
+      <c r="H7" s="83" t="n">
+        <v>24</v>
+      </c>
+      <c r="I7" s="83" t="inlineStr">
+        <is>
+          <t>لكل فرد</t>
+        </is>
+      </c>
+      <c r="J7" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
+      <c r="K7" s="83" t="inlineStr">
+        <is>
+          <t>بعد كل رحلة</t>
+        </is>
+      </c>
+      <c r="L7" s="83" t="inlineStr">
+        <is>
+          <t>كاش</t>
+        </is>
+      </c>
+      <c r="M7" s="83" t="inlineStr">
+        <is>
+          <t>خصم</t>
+        </is>
+      </c>
       <c r="N7" s="83" t="inlineStr"/>
       <c r="O7" s="82" t="inlineStr">
         <is>
@@ -6815,25 +7029,25 @@
     <mergeCell ref="A1:O1"/>
   </mergeCells>
   <dataValidations count="7">
-    <dataValidation sqref="C3:C17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C3:C17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"مراكب,كواد/باجي/سفاري,غوص/سنوركل,عروض وترفيه,نقل/عربيات,مرشدين,طيران/رحلات بعيدة,أخرى"</formula1>
     </dataValidation>
-    <dataValidation sqref="G3:G17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G3:G17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"واتساب,تليفون,إيميل,بيجي المكتب"</formula1>
     </dataValidation>
-    <dataValidation sqref="I3:I17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I3:I17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"سعر ثابت للرحلة,لكل فرد,لكل وحدة (باجي/مركب/عربية),نسبة من سعر البيع"</formula1>
     </dataValidation>
-    <dataValidation sqref="J3:J17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J3:J17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"جنيه,يورو,دولار"</formula1>
     </dataValidation>
-    <dataValidation sqref="K3:K17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K3:K17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"بعد كل رحلة,آخر الأسبوع,آخر الشهر,غير كده (اكتب في الملاحظات)"</formula1>
     </dataValidation>
-    <dataValidation sqref="L3:L17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L3:L17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"كاش,تحويل بنكي,إنستاباي,محفظة إلكترونية"</formula1>
     </dataValidation>
-    <dataValidation sqref="O3:O17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="O3:O17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"ناقص,اتملى,محتاج مراجعة,مش محتاجينه"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6934,17 +7148,29 @@
         </is>
       </c>
       <c r="B3" s="83" t="inlineStr"/>
-      <c r="C3" s="83" t="inlineStr"/>
+      <c r="C3" s="83" t="n">
+        <v>1100</v>
+      </c>
       <c r="D3" s="83" t="inlineStr"/>
-      <c r="E3" s="83" t="inlineStr"/>
+      <c r="E3" s="83" t="inlineStr">
+        <is>
+          <t>بتش بجي</t>
+        </is>
+      </c>
       <c r="F3" s="83" t="inlineStr"/>
-      <c r="G3" s="83" t="inlineStr"/>
+      <c r="G3" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
       <c r="H3" s="83" t="inlineStr">
         <is>
-          <t>كل السنة</t>
-        </is>
-      </c>
-      <c r="I3" s="83" t="inlineStr"/>
+          <t>موسم عادي</t>
+        </is>
+      </c>
+      <c r="I3" s="84" t="n">
+        <v>46032</v>
+      </c>
       <c r="J3" s="83" t="inlineStr"/>
       <c r="K3" s="83" t="inlineStr"/>
     </row>
@@ -6955,17 +7181,29 @@
         </is>
       </c>
       <c r="B4" s="83" t="inlineStr"/>
-      <c r="C4" s="83" t="inlineStr"/>
+      <c r="C4" s="83" t="n">
+        <v>600</v>
+      </c>
       <c r="D4" s="83" t="inlineStr"/>
-      <c r="E4" s="83" t="inlineStr"/>
+      <c r="E4" s="83" t="inlineStr">
+        <is>
+          <t>بتش بجي</t>
+        </is>
+      </c>
       <c r="F4" s="83" t="inlineStr"/>
-      <c r="G4" s="83" t="inlineStr"/>
+      <c r="G4" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
       <c r="H4" s="83" t="inlineStr">
         <is>
-          <t>كل السنة</t>
-        </is>
-      </c>
-      <c r="I4" s="83" t="inlineStr"/>
+          <t>موسم عادي</t>
+        </is>
+      </c>
+      <c r="I4" s="84" t="n">
+        <v>46032</v>
+      </c>
       <c r="J4" s="83" t="inlineStr"/>
       <c r="K4" s="83" t="inlineStr"/>
     </row>
@@ -6976,17 +7214,29 @@
         </is>
       </c>
       <c r="B5" s="83" t="inlineStr"/>
-      <c r="C5" s="83" t="inlineStr"/>
+      <c r="C5" s="83" t="n">
+        <v>1200</v>
+      </c>
       <c r="D5" s="83" t="inlineStr"/>
-      <c r="E5" s="83" t="inlineStr"/>
+      <c r="E5" s="83" t="inlineStr">
+        <is>
+          <t>كار بجي +جمل</t>
+        </is>
+      </c>
       <c r="F5" s="83" t="inlineStr"/>
-      <c r="G5" s="83" t="inlineStr"/>
+      <c r="G5" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
       <c r="H5" s="83" t="inlineStr">
         <is>
-          <t>كل السنة</t>
-        </is>
-      </c>
-      <c r="I5" s="83" t="inlineStr"/>
+          <t>موسم عادي</t>
+        </is>
+      </c>
+      <c r="I5" s="84" t="n">
+        <v>46032</v>
+      </c>
       <c r="J5" s="83" t="inlineStr"/>
       <c r="K5" s="83" t="inlineStr"/>
     </row>
@@ -6997,17 +7247,29 @@
         </is>
       </c>
       <c r="B6" s="83" t="inlineStr"/>
-      <c r="C6" s="83" t="inlineStr"/>
+      <c r="C6" s="83" t="n">
+        <v>650</v>
+      </c>
       <c r="D6" s="83" t="inlineStr"/>
-      <c r="E6" s="83" t="inlineStr"/>
+      <c r="E6" s="83" t="inlineStr">
+        <is>
+          <t>عشاء +جمل</t>
+        </is>
+      </c>
       <c r="F6" s="83" t="inlineStr"/>
-      <c r="G6" s="83" t="inlineStr"/>
+      <c r="G6" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
       <c r="H6" s="83" t="inlineStr">
         <is>
-          <t>كل السنة</t>
-        </is>
-      </c>
-      <c r="I6" s="83" t="inlineStr"/>
+          <t>موسم عادي</t>
+        </is>
+      </c>
+      <c r="I6" s="84" t="n">
+        <v>46032</v>
+      </c>
       <c r="J6" s="83" t="inlineStr"/>
       <c r="K6" s="83" t="inlineStr"/>
     </row>
@@ -7018,19 +7280,35 @@
         </is>
       </c>
       <c r="B7" s="83" t="inlineStr"/>
-      <c r="C7" s="83" t="inlineStr"/>
+      <c r="C7" s="83" t="n">
+        <v>800</v>
+      </c>
       <c r="D7" s="83" t="inlineStr"/>
-      <c r="E7" s="83" t="inlineStr"/>
+      <c r="E7" s="83" t="inlineStr">
+        <is>
+          <t>شامل غداء</t>
+        </is>
+      </c>
       <c r="F7" s="83" t="inlineStr"/>
-      <c r="G7" s="83" t="inlineStr"/>
+      <c r="G7" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
       <c r="H7" s="83" t="inlineStr">
         <is>
-          <t>كل السنة</t>
-        </is>
-      </c>
-      <c r="I7" s="83" t="inlineStr"/>
+          <t>موسم عادي</t>
+        </is>
+      </c>
+      <c r="I7" s="84" t="n">
+        <v>46032</v>
+      </c>
       <c r="J7" s="83" t="inlineStr"/>
-      <c r="K7" s="83" t="inlineStr"/>
+      <c r="K7" s="83" t="inlineStr">
+        <is>
+          <t>جيب +جمل +بتش بجي</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="82" t="inlineStr">
@@ -7039,17 +7317,29 @@
         </is>
       </c>
       <c r="B8" s="83" t="inlineStr"/>
-      <c r="C8" s="83" t="inlineStr"/>
+      <c r="C8" s="83" t="n">
+        <v>1250</v>
+      </c>
       <c r="D8" s="83" t="inlineStr"/>
-      <c r="E8" s="83" t="inlineStr"/>
+      <c r="E8" s="83" t="inlineStr">
+        <is>
+          <t>transafer</t>
+        </is>
+      </c>
       <c r="F8" s="83" t="inlineStr"/>
-      <c r="G8" s="83" t="inlineStr"/>
+      <c r="G8" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
       <c r="H8" s="83" t="inlineStr">
         <is>
-          <t>كل السنة</t>
-        </is>
-      </c>
-      <c r="I8" s="83" t="inlineStr"/>
+          <t>موسم عادي</t>
+        </is>
+      </c>
+      <c r="I8" s="84" t="n">
+        <v>46305</v>
+      </c>
       <c r="J8" s="83" t="inlineStr"/>
       <c r="K8" s="83" t="inlineStr"/>
     </row>
@@ -7060,19 +7350,35 @@
         </is>
       </c>
       <c r="B9" s="83" t="inlineStr"/>
-      <c r="C9" s="83" t="inlineStr"/>
+      <c r="C9" s="83" t="n">
+        <v>1300</v>
+      </c>
       <c r="D9" s="83" t="inlineStr"/>
-      <c r="E9" s="83" t="inlineStr"/>
+      <c r="E9" s="83" t="inlineStr">
+        <is>
+          <t>شامل غداء</t>
+        </is>
+      </c>
       <c r="F9" s="83" t="inlineStr"/>
-      <c r="G9" s="83" t="inlineStr"/>
+      <c r="G9" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
       <c r="H9" s="83" t="inlineStr">
         <is>
-          <t>كل السنة</t>
-        </is>
-      </c>
-      <c r="I9" s="83" t="inlineStr"/>
+          <t>موسم عادي</t>
+        </is>
+      </c>
+      <c r="I9" s="84" t="n">
+        <v>46296</v>
+      </c>
       <c r="J9" s="83" t="inlineStr"/>
-      <c r="K9" s="83" t="inlineStr"/>
+      <c r="K9" s="83" t="inlineStr">
+        <is>
+          <t>غداء سوفت درينك</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="82" t="inlineStr">
@@ -7081,17 +7387,29 @@
         </is>
       </c>
       <c r="B10" s="83" t="inlineStr"/>
-      <c r="C10" s="83" t="inlineStr"/>
+      <c r="C10" s="83" t="n">
+        <v>1000</v>
+      </c>
       <c r="D10" s="83" t="inlineStr"/>
-      <c r="E10" s="83" t="inlineStr"/>
+      <c r="E10" s="83" t="inlineStr">
+        <is>
+          <t>شامل غداء</t>
+        </is>
+      </c>
       <c r="F10" s="83" t="inlineStr"/>
-      <c r="G10" s="83" t="inlineStr"/>
+      <c r="G10" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
       <c r="H10" s="83" t="inlineStr">
         <is>
-          <t>كل السنة</t>
-        </is>
-      </c>
-      <c r="I10" s="83" t="inlineStr"/>
+          <t>موسم عادي</t>
+        </is>
+      </c>
+      <c r="I10" s="84" t="n">
+        <v>46032</v>
+      </c>
       <c r="J10" s="83" t="inlineStr"/>
       <c r="K10" s="83" t="inlineStr"/>
     </row>
@@ -7102,17 +7420,29 @@
         </is>
       </c>
       <c r="B11" s="83" t="inlineStr"/>
-      <c r="C11" s="83" t="inlineStr"/>
+      <c r="C11" s="83" t="n">
+        <v>350</v>
+      </c>
       <c r="D11" s="83" t="inlineStr"/>
-      <c r="E11" s="83" t="inlineStr"/>
+      <c r="E11" s="83" t="inlineStr">
+        <is>
+          <t>transafer</t>
+        </is>
+      </c>
       <c r="F11" s="83" t="inlineStr"/>
-      <c r="G11" s="83" t="inlineStr"/>
+      <c r="G11" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
       <c r="H11" s="83" t="inlineStr">
         <is>
-          <t>كل السنة</t>
-        </is>
-      </c>
-      <c r="I11" s="83" t="inlineStr"/>
+          <t>موسم عالي</t>
+        </is>
+      </c>
+      <c r="I11" s="84" t="n">
+        <v>46031</v>
+      </c>
       <c r="J11" s="83" t="inlineStr"/>
       <c r="K11" s="83" t="inlineStr"/>
     </row>
@@ -7123,17 +7453,29 @@
         </is>
       </c>
       <c r="B12" s="83" t="inlineStr"/>
-      <c r="C12" s="83" t="inlineStr"/>
+      <c r="C12" s="83" t="n">
+        <v>17500</v>
+      </c>
       <c r="D12" s="83" t="inlineStr"/>
-      <c r="E12" s="83" t="inlineStr"/>
+      <c r="E12" s="83" t="inlineStr">
+        <is>
+          <t>3 day 4 day</t>
+        </is>
+      </c>
       <c r="F12" s="83" t="inlineStr"/>
-      <c r="G12" s="83" t="inlineStr"/>
+      <c r="G12" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
       <c r="H12" s="83" t="inlineStr">
         <is>
-          <t>كل السنة</t>
-        </is>
-      </c>
-      <c r="I12" s="83" t="inlineStr"/>
+          <t>موسم عادي</t>
+        </is>
+      </c>
+      <c r="I12" s="84" t="n">
+        <v>46028</v>
+      </c>
       <c r="J12" s="83" t="inlineStr"/>
       <c r="K12" s="83" t="inlineStr"/>
     </row>
@@ -7144,17 +7486,29 @@
         </is>
       </c>
       <c r="B13" s="83" t="inlineStr"/>
-      <c r="C13" s="83" t="inlineStr"/>
+      <c r="C13" s="83" t="n">
+        <v>2750</v>
+      </c>
       <c r="D13" s="83" t="inlineStr"/>
-      <c r="E13" s="83" t="inlineStr"/>
+      <c r="E13" s="83" t="inlineStr">
+        <is>
+          <t>شامل غداء</t>
+        </is>
+      </c>
       <c r="F13" s="83" t="inlineStr"/>
-      <c r="G13" s="83" t="inlineStr"/>
+      <c r="G13" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
       <c r="H13" s="83" t="inlineStr">
         <is>
-          <t>كل السنة</t>
-        </is>
-      </c>
-      <c r="I13" s="83" t="inlineStr"/>
+          <t>موسم عادي</t>
+        </is>
+      </c>
+      <c r="I13" s="84" t="n">
+        <v>46028</v>
+      </c>
       <c r="J13" s="83" t="inlineStr"/>
       <c r="K13" s="83" t="inlineStr"/>
     </row>
@@ -7165,17 +7519,29 @@
         </is>
       </c>
       <c r="B14" s="83" t="inlineStr"/>
-      <c r="C14" s="83" t="inlineStr"/>
+      <c r="C14" s="83" t="n">
+        <v>800</v>
+      </c>
       <c r="D14" s="83" t="inlineStr"/>
-      <c r="E14" s="83" t="inlineStr"/>
+      <c r="E14" s="83" t="inlineStr">
+        <is>
+          <t>transafer</t>
+        </is>
+      </c>
       <c r="F14" s="83" t="inlineStr"/>
-      <c r="G14" s="83" t="inlineStr"/>
+      <c r="G14" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
       <c r="H14" s="83" t="inlineStr">
         <is>
-          <t>كل السنة</t>
-        </is>
-      </c>
-      <c r="I14" s="83" t="inlineStr"/>
+          <t>موسم عادي</t>
+        </is>
+      </c>
+      <c r="I14" s="84" t="n">
+        <v>46023</v>
+      </c>
       <c r="J14" s="83" t="inlineStr"/>
       <c r="K14" s="83" t="inlineStr"/>
     </row>
@@ -7186,17 +7552,29 @@
         </is>
       </c>
       <c r="B15" s="83" t="inlineStr"/>
-      <c r="C15" s="83" t="inlineStr"/>
+      <c r="C15" s="83" t="n">
+        <v>800</v>
+      </c>
       <c r="D15" s="83" t="inlineStr"/>
-      <c r="E15" s="83" t="inlineStr"/>
+      <c r="E15" s="83" t="inlineStr">
+        <is>
+          <t>transafer</t>
+        </is>
+      </c>
       <c r="F15" s="83" t="inlineStr"/>
-      <c r="G15" s="83" t="inlineStr"/>
+      <c r="G15" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
       <c r="H15" s="83" t="inlineStr">
         <is>
-          <t>كل السنة</t>
-        </is>
-      </c>
-      <c r="I15" s="83" t="inlineStr"/>
+          <t>موسم عادي</t>
+        </is>
+      </c>
+      <c r="I15" s="84" t="n">
+        <v>46209</v>
+      </c>
       <c r="J15" s="83" t="inlineStr"/>
       <c r="K15" s="83" t="inlineStr"/>
     </row>
@@ -7207,19 +7585,37 @@
         </is>
       </c>
       <c r="B16" s="83" t="inlineStr"/>
-      <c r="C16" s="83" t="inlineStr"/>
+      <c r="C16" s="83" t="inlineStr">
+        <is>
+          <t>600/800</t>
+        </is>
+      </c>
       <c r="D16" s="83" t="inlineStr"/>
-      <c r="E16" s="83" t="inlineStr"/>
+      <c r="E16" s="83" t="inlineStr">
+        <is>
+          <t>transafer</t>
+        </is>
+      </c>
       <c r="F16" s="83" t="inlineStr"/>
-      <c r="G16" s="83" t="inlineStr"/>
+      <c r="G16" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
       <c r="H16" s="83" t="inlineStr">
         <is>
-          <t>كل السنة</t>
-        </is>
-      </c>
-      <c r="I16" s="83" t="inlineStr"/>
+          <t>موسم عادي</t>
+        </is>
+      </c>
+      <c r="I16" s="84" t="n">
+        <v>46028</v>
+      </c>
       <c r="J16" s="83" t="inlineStr"/>
-      <c r="K16" s="83" t="inlineStr"/>
+      <c r="K16" s="83" t="inlineStr">
+        <is>
+          <t>snigel 600 doubel 800</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="82" t="inlineStr">
@@ -7228,19 +7624,35 @@
         </is>
       </c>
       <c r="B17" s="83" t="inlineStr"/>
-      <c r="C17" s="83" t="inlineStr"/>
+      <c r="C17" s="83" t="n">
+        <v>5000</v>
+      </c>
       <c r="D17" s="83" t="inlineStr"/>
-      <c r="E17" s="83" t="inlineStr"/>
+      <c r="E17" s="83" t="inlineStr">
+        <is>
+          <t>transafer</t>
+        </is>
+      </c>
       <c r="F17" s="83" t="inlineStr"/>
-      <c r="G17" s="83" t="inlineStr"/>
+      <c r="G17" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
       <c r="H17" s="83" t="inlineStr">
         <is>
-          <t>كل السنة</t>
-        </is>
-      </c>
-      <c r="I17" s="83" t="inlineStr"/>
+          <t>موسم عادي</t>
+        </is>
+      </c>
+      <c r="I17" s="84" t="n">
+        <v>46028</v>
+      </c>
       <c r="J17" s="83" t="inlineStr"/>
-      <c r="K17" s="83" t="inlineStr"/>
+      <c r="K17" s="83" t="inlineStr">
+        <is>
+          <t>سعر الساعه 5000</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="82" t="inlineStr">
@@ -7249,17 +7661,29 @@
         </is>
       </c>
       <c r="B18" s="83" t="inlineStr"/>
-      <c r="C18" s="83" t="inlineStr"/>
+      <c r="C18" s="83" t="n">
+        <v>1450</v>
+      </c>
       <c r="D18" s="83" t="inlineStr"/>
-      <c r="E18" s="83" t="inlineStr"/>
+      <c r="E18" s="83" t="inlineStr">
+        <is>
+          <t>transafer</t>
+        </is>
+      </c>
       <c r="F18" s="83" t="inlineStr"/>
-      <c r="G18" s="83" t="inlineStr"/>
+      <c r="G18" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
       <c r="H18" s="83" t="inlineStr">
         <is>
-          <t>كل السنة</t>
-        </is>
-      </c>
-      <c r="I18" s="83" t="inlineStr"/>
+          <t>موسم عادي</t>
+        </is>
+      </c>
+      <c r="I18" s="84" t="n">
+        <v>46028</v>
+      </c>
       <c r="J18" s="83" t="inlineStr"/>
       <c r="K18" s="83" t="inlineStr"/>
     </row>
@@ -7270,19 +7694,35 @@
         </is>
       </c>
       <c r="B19" s="83" t="inlineStr"/>
-      <c r="C19" s="83" t="inlineStr"/>
+      <c r="C19" s="83" t="n">
+        <v>1300</v>
+      </c>
       <c r="D19" s="83" t="inlineStr"/>
-      <c r="E19" s="83" t="inlineStr"/>
+      <c r="E19" s="83" t="inlineStr">
+        <is>
+          <t>transafer</t>
+        </is>
+      </c>
       <c r="F19" s="83" t="inlineStr"/>
-      <c r="G19" s="83" t="inlineStr"/>
+      <c r="G19" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
       <c r="H19" s="83" t="inlineStr">
         <is>
-          <t>كل السنة</t>
-        </is>
-      </c>
-      <c r="I19" s="83" t="inlineStr"/>
+          <t>موسم عادي</t>
+        </is>
+      </c>
+      <c r="I19" s="84" t="n">
+        <v>46029</v>
+      </c>
       <c r="J19" s="83" t="inlineStr"/>
-      <c r="K19" s="83" t="inlineStr"/>
+      <c r="K19" s="83" t="inlineStr">
+        <is>
+          <t>غداء سوفت درينك</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="82" t="inlineStr">
@@ -7291,17 +7731,29 @@
         </is>
       </c>
       <c r="B20" s="83" t="inlineStr"/>
-      <c r="C20" s="83" t="inlineStr"/>
+      <c r="C20" s="83" t="n">
+        <v>800</v>
+      </c>
       <c r="D20" s="83" t="inlineStr"/>
-      <c r="E20" s="83" t="inlineStr"/>
+      <c r="E20" s="83" t="inlineStr">
+        <is>
+          <t>transafer</t>
+        </is>
+      </c>
       <c r="F20" s="83" t="inlineStr"/>
-      <c r="G20" s="83" t="inlineStr"/>
+      <c r="G20" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
       <c r="H20" s="83" t="inlineStr">
         <is>
-          <t>كل السنة</t>
-        </is>
-      </c>
-      <c r="I20" s="83" t="inlineStr"/>
+          <t>موسم عادي</t>
+        </is>
+      </c>
+      <c r="I20" s="84" t="n">
+        <v>46027</v>
+      </c>
       <c r="J20" s="83" t="inlineStr"/>
       <c r="K20" s="83" t="inlineStr"/>
     </row>
@@ -7312,17 +7764,29 @@
         </is>
       </c>
       <c r="B21" s="83" t="inlineStr"/>
-      <c r="C21" s="83" t="inlineStr"/>
+      <c r="C21" s="83" t="n">
+        <v>2000</v>
+      </c>
       <c r="D21" s="83" t="inlineStr"/>
-      <c r="E21" s="83" t="inlineStr"/>
+      <c r="E21" s="83" t="inlineStr">
+        <is>
+          <t>transafer</t>
+        </is>
+      </c>
       <c r="F21" s="83" t="inlineStr"/>
-      <c r="G21" s="83" t="inlineStr"/>
+      <c r="G21" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
       <c r="H21" s="83" t="inlineStr">
         <is>
-          <t>كل السنة</t>
-        </is>
-      </c>
-      <c r="I21" s="83" t="inlineStr"/>
+          <t>موسم عادي</t>
+        </is>
+      </c>
+      <c r="I21" s="84" t="n">
+        <v>46023</v>
+      </c>
       <c r="J21" s="83" t="inlineStr"/>
       <c r="K21" s="83" t="inlineStr"/>
     </row>
@@ -7333,17 +7797,29 @@
         </is>
       </c>
       <c r="B22" s="83" t="inlineStr"/>
-      <c r="C22" s="83" t="inlineStr"/>
+      <c r="C22" s="83" t="n">
+        <v>12000</v>
+      </c>
       <c r="D22" s="83" t="inlineStr"/>
-      <c r="E22" s="83" t="inlineStr"/>
+      <c r="E22" s="83" t="inlineStr">
+        <is>
+          <t>transafer</t>
+        </is>
+      </c>
       <c r="F22" s="83" t="inlineStr"/>
-      <c r="G22" s="83" t="inlineStr"/>
+      <c r="G22" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
       <c r="H22" s="83" t="inlineStr">
         <is>
-          <t>كل السنة</t>
-        </is>
-      </c>
-      <c r="I22" s="83" t="inlineStr"/>
+          <t>موسم عادي</t>
+        </is>
+      </c>
+      <c r="I22" s="84" t="n">
+        <v>46023</v>
+      </c>
       <c r="J22" s="83" t="inlineStr"/>
       <c r="K22" s="83" t="inlineStr"/>
     </row>
@@ -7354,17 +7830,29 @@
         </is>
       </c>
       <c r="B23" s="83" t="inlineStr"/>
-      <c r="C23" s="83" t="inlineStr"/>
+      <c r="C23" s="83" t="n">
+        <v>1300</v>
+      </c>
       <c r="D23" s="83" t="inlineStr"/>
-      <c r="E23" s="83" t="inlineStr"/>
+      <c r="E23" s="83" t="inlineStr">
+        <is>
+          <t>transafer</t>
+        </is>
+      </c>
       <c r="F23" s="83" t="inlineStr"/>
-      <c r="G23" s="83" t="inlineStr"/>
+      <c r="G23" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
       <c r="H23" s="83" t="inlineStr">
         <is>
-          <t>كل السنة</t>
-        </is>
-      </c>
-      <c r="I23" s="83" t="inlineStr"/>
+          <t>موسم عادي</t>
+        </is>
+      </c>
+      <c r="I23" s="84" t="n">
+        <v>46023</v>
+      </c>
       <c r="J23" s="83" t="inlineStr"/>
       <c r="K23" s="83" t="inlineStr"/>
     </row>
@@ -7375,17 +7863,29 @@
         </is>
       </c>
       <c r="B24" s="83" t="inlineStr"/>
-      <c r="C24" s="83" t="inlineStr"/>
+      <c r="C24" s="83" t="n">
+        <v>13000</v>
+      </c>
       <c r="D24" s="83" t="inlineStr"/>
-      <c r="E24" s="83" t="inlineStr"/>
+      <c r="E24" s="83" t="inlineStr">
+        <is>
+          <t>transafer</t>
+        </is>
+      </c>
       <c r="F24" s="83" t="inlineStr"/>
-      <c r="G24" s="83" t="inlineStr"/>
+      <c r="G24" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
       <c r="H24" s="83" t="inlineStr">
         <is>
-          <t>كل السنة</t>
-        </is>
-      </c>
-      <c r="I24" s="83" t="inlineStr"/>
+          <t>موسم عادي</t>
+        </is>
+      </c>
+      <c r="I24" s="84" t="n">
+        <v>46023</v>
+      </c>
       <c r="J24" s="83" t="inlineStr"/>
       <c r="K24" s="83" t="inlineStr"/>
     </row>
@@ -7396,17 +7896,29 @@
         </is>
       </c>
       <c r="B25" s="83" t="inlineStr"/>
-      <c r="C25" s="83" t="inlineStr"/>
+      <c r="C25" s="83" t="n">
+        <v>1400</v>
+      </c>
       <c r="D25" s="83" t="inlineStr"/>
-      <c r="E25" s="83" t="inlineStr"/>
+      <c r="E25" s="83" t="inlineStr">
+        <is>
+          <t>transafer</t>
+        </is>
+      </c>
       <c r="F25" s="83" t="inlineStr"/>
-      <c r="G25" s="83" t="inlineStr"/>
+      <c r="G25" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
       <c r="H25" s="83" t="inlineStr">
         <is>
-          <t>كل السنة</t>
-        </is>
-      </c>
-      <c r="I25" s="83" t="inlineStr"/>
+          <t>موسم عادي</t>
+        </is>
+      </c>
+      <c r="I25" s="84" t="n">
+        <v>46023</v>
+      </c>
       <c r="J25" s="83" t="inlineStr"/>
       <c r="K25" s="83" t="inlineStr"/>
     </row>
@@ -7417,17 +7929,29 @@
         </is>
       </c>
       <c r="B26" s="83" t="inlineStr"/>
-      <c r="C26" s="83" t="inlineStr"/>
+      <c r="C26" s="83" t="n">
+        <v>1700</v>
+      </c>
       <c r="D26" s="83" t="inlineStr"/>
-      <c r="E26" s="83" t="inlineStr"/>
+      <c r="E26" s="83" t="inlineStr">
+        <is>
+          <t>transafer</t>
+        </is>
+      </c>
       <c r="F26" s="83" t="inlineStr"/>
-      <c r="G26" s="83" t="inlineStr"/>
+      <c r="G26" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
       <c r="H26" s="83" t="inlineStr">
         <is>
-          <t>كل السنة</t>
-        </is>
-      </c>
-      <c r="I26" s="83" t="inlineStr"/>
+          <t>موسم عادي</t>
+        </is>
+      </c>
+      <c r="I26" s="84" t="n">
+        <v>46023</v>
+      </c>
       <c r="J26" s="83" t="inlineStr"/>
       <c r="K26" s="83" t="inlineStr"/>
     </row>
@@ -7438,17 +7962,29 @@
         </is>
       </c>
       <c r="B27" s="83" t="inlineStr"/>
-      <c r="C27" s="83" t="inlineStr"/>
+      <c r="C27" s="83" t="n">
+        <v>700</v>
+      </c>
       <c r="D27" s="83" t="inlineStr"/>
-      <c r="E27" s="83" t="inlineStr"/>
+      <c r="E27" s="83" t="inlineStr">
+        <is>
+          <t>transafer</t>
+        </is>
+      </c>
       <c r="F27" s="83" t="inlineStr"/>
-      <c r="G27" s="83" t="inlineStr"/>
+      <c r="G27" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
       <c r="H27" s="83" t="inlineStr">
         <is>
-          <t>كل السنة</t>
-        </is>
-      </c>
-      <c r="I27" s="83" t="inlineStr"/>
+          <t>موسم عادي</t>
+        </is>
+      </c>
+      <c r="I27" s="84" t="n">
+        <v>46023</v>
+      </c>
       <c r="J27" s="83" t="inlineStr"/>
       <c r="K27" s="83" t="inlineStr"/>
     </row>
@@ -7459,17 +7995,29 @@
         </is>
       </c>
       <c r="B28" s="83" t="inlineStr"/>
-      <c r="C28" s="83" t="inlineStr"/>
+      <c r="C28" s="83" t="n">
+        <v>3550</v>
+      </c>
       <c r="D28" s="83" t="inlineStr"/>
-      <c r="E28" s="83" t="inlineStr"/>
+      <c r="E28" s="83" t="inlineStr">
+        <is>
+          <t>transafer</t>
+        </is>
+      </c>
       <c r="F28" s="83" t="inlineStr"/>
-      <c r="G28" s="83" t="inlineStr"/>
+      <c r="G28" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
       <c r="H28" s="83" t="inlineStr">
         <is>
-          <t>كل السنة</t>
-        </is>
-      </c>
-      <c r="I28" s="83" t="inlineStr"/>
+          <t>موسم عادي</t>
+        </is>
+      </c>
+      <c r="I28" s="84" t="n">
+        <v>46023</v>
+      </c>
       <c r="J28" s="83" t="inlineStr"/>
       <c r="K28" s="83" t="inlineStr"/>
     </row>
@@ -7480,17 +8028,29 @@
         </is>
       </c>
       <c r="B29" s="83" t="inlineStr"/>
-      <c r="C29" s="83" t="inlineStr"/>
+      <c r="C29" s="83" t="n">
+        <v>600</v>
+      </c>
       <c r="D29" s="83" t="inlineStr"/>
-      <c r="E29" s="83" t="inlineStr"/>
+      <c r="E29" s="83" t="inlineStr">
+        <is>
+          <t>transafer</t>
+        </is>
+      </c>
       <c r="F29" s="83" t="inlineStr"/>
-      <c r="G29" s="83" t="inlineStr"/>
+      <c r="G29" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
       <c r="H29" s="83" t="inlineStr">
         <is>
-          <t>كل السنة</t>
-        </is>
-      </c>
-      <c r="I29" s="83" t="inlineStr"/>
+          <t>موسم عادي</t>
+        </is>
+      </c>
+      <c r="I29" s="84" t="n">
+        <v>46023</v>
+      </c>
       <c r="J29" s="83" t="inlineStr"/>
       <c r="K29" s="83" t="inlineStr"/>
     </row>
@@ -7499,10 +8059,10 @@
     <mergeCell ref="A1:K1"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="G3:G29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G3:G29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"جنيه,يورو,دولار"</formula1>
     </dataValidation>
-    <dataValidation sqref="H3:H29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H3:H29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"كل السنة,موسم عالي,موسم عادي"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7602,18 +8162,46 @@
           <t>D01</t>
         </is>
       </c>
-      <c r="B3" s="83" t="inlineStr"/>
-      <c r="C3" s="83" t="inlineStr"/>
-      <c r="D3" s="83" t="inlineStr"/>
-      <c r="E3" s="83" t="inlineStr"/>
-      <c r="F3" s="83" t="inlineStr"/>
-      <c r="G3" s="83" t="inlineStr"/>
-      <c r="H3" s="83" t="inlineStr"/>
-      <c r="I3" s="83" t="inlineStr"/>
+      <c r="B3" s="83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">عمرو </t>
+        </is>
+      </c>
+      <c r="C3" s="83" t="n">
+        <v>1028215951</v>
+      </c>
+      <c r="D3" s="83" t="inlineStr">
+        <is>
+          <t>بالمشوار</t>
+        </is>
+      </c>
+      <c r="E3" s="83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">حسب التشغيله </t>
+        </is>
+      </c>
+      <c r="F3" s="83" t="inlineStr">
+        <is>
+          <t>مشوار</t>
+        </is>
+      </c>
+      <c r="G3" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
+      <c r="H3" s="83" t="n">
+        <v>2027</v>
+      </c>
+      <c r="I3" s="83" t="inlineStr">
+        <is>
+          <t>شري اريزو</t>
+        </is>
+      </c>
       <c r="J3" s="83" t="inlineStr"/>
       <c r="K3" s="82" t="inlineStr">
         <is>
-          <t>ناقص</t>
+          <t>اتملى</t>
         </is>
       </c>
     </row>
@@ -7623,14 +8211,42 @@
           <t>D02</t>
         </is>
       </c>
-      <c r="B4" s="83" t="inlineStr"/>
-      <c r="C4" s="83" t="inlineStr"/>
-      <c r="D4" s="83" t="inlineStr"/>
-      <c r="E4" s="83" t="inlineStr"/>
-      <c r="F4" s="83" t="inlineStr"/>
-      <c r="G4" s="83" t="inlineStr"/>
-      <c r="H4" s="83" t="inlineStr"/>
-      <c r="I4" s="83" t="inlineStr"/>
+      <c r="B4" s="83" t="inlineStr">
+        <is>
+          <t>ياسر</t>
+        </is>
+      </c>
+      <c r="C4" s="83" t="n">
+        <v>1000651421</v>
+      </c>
+      <c r="D4" s="83" t="inlineStr">
+        <is>
+          <t>بالمشوار</t>
+        </is>
+      </c>
+      <c r="E4" s="83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">حسب التشغيله </t>
+        </is>
+      </c>
+      <c r="F4" s="83" t="inlineStr">
+        <is>
+          <t>مشوار</t>
+        </is>
+      </c>
+      <c r="G4" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
+      <c r="H4" s="83" t="n">
+        <v>2027</v>
+      </c>
+      <c r="I4" s="83" t="inlineStr">
+        <is>
+          <t>هاي اس</t>
+        </is>
+      </c>
       <c r="J4" s="83" t="inlineStr"/>
       <c r="K4" s="82" t="inlineStr">
         <is>
@@ -7644,14 +8260,42 @@
           <t>D03</t>
         </is>
       </c>
-      <c r="B5" s="83" t="inlineStr"/>
-      <c r="C5" s="83" t="inlineStr"/>
-      <c r="D5" s="83" t="inlineStr"/>
-      <c r="E5" s="83" t="inlineStr"/>
-      <c r="F5" s="83" t="inlineStr"/>
-      <c r="G5" s="83" t="inlineStr"/>
-      <c r="H5" s="83" t="inlineStr"/>
-      <c r="I5" s="83" t="inlineStr"/>
+      <c r="B5" s="83" t="inlineStr">
+        <is>
+          <t>حسام</t>
+        </is>
+      </c>
+      <c r="C5" s="83" t="n">
+        <v>1001810343</v>
+      </c>
+      <c r="D5" s="83" t="inlineStr">
+        <is>
+          <t>بالمشوار</t>
+        </is>
+      </c>
+      <c r="E5" s="83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">حسب التشغيله </t>
+        </is>
+      </c>
+      <c r="F5" s="83" t="inlineStr">
+        <is>
+          <t>مشوار</t>
+        </is>
+      </c>
+      <c r="G5" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
+      <c r="H5" s="83" t="n">
+        <v>2028</v>
+      </c>
+      <c r="I5" s="83" t="inlineStr">
+        <is>
+          <t>شري تيجو 8</t>
+        </is>
+      </c>
       <c r="J5" s="83" t="inlineStr"/>
       <c r="K5" s="82" t="inlineStr">
         <is>
@@ -7665,14 +8309,42 @@
           <t>D04</t>
         </is>
       </c>
-      <c r="B6" s="83" t="inlineStr"/>
-      <c r="C6" s="83" t="inlineStr"/>
-      <c r="D6" s="83" t="inlineStr"/>
-      <c r="E6" s="83" t="inlineStr"/>
-      <c r="F6" s="83" t="inlineStr"/>
-      <c r="G6" s="83" t="inlineStr"/>
-      <c r="H6" s="83" t="inlineStr"/>
-      <c r="I6" s="83" t="inlineStr"/>
+      <c r="B6" s="83" t="inlineStr">
+        <is>
+          <t>سعد</t>
+        </is>
+      </c>
+      <c r="C6" s="83" t="n">
+        <v>1014772369</v>
+      </c>
+      <c r="D6" s="83" t="inlineStr">
+        <is>
+          <t>بالمشوار</t>
+        </is>
+      </c>
+      <c r="E6" s="83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">حسب التشغيله </t>
+        </is>
+      </c>
+      <c r="F6" s="83" t="inlineStr">
+        <is>
+          <t>مشوار</t>
+        </is>
+      </c>
+      <c r="G6" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
+      <c r="H6" s="83" t="n">
+        <v>2027</v>
+      </c>
+      <c r="I6" s="83" t="inlineStr">
+        <is>
+          <t>نيسان صنس</t>
+        </is>
+      </c>
       <c r="J6" s="83" t="inlineStr"/>
       <c r="K6" s="82" t="inlineStr">
         <is>
@@ -7811,16 +8483,16 @@
     <mergeCell ref="A1:K1"/>
   </mergeCells>
   <dataValidations count="4">
-    <dataValidation sqref="D3:D12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D3:D12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"موظف بمرتب,بالمشوار,باليوم,من مورد نقل"</formula1>
     </dataValidation>
-    <dataValidation sqref="F3:F12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F3:F12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"شهر,مشوار,يوم,رحلة"</formula1>
     </dataValidation>
-    <dataValidation sqref="G3:G12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G3:G12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"جنيه,يورو"</formula1>
     </dataValidation>
-    <dataValidation sqref="K3:K12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K3:K12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"ناقص,اتملى,محتاج مراجعة,مش محتاجينه"</formula1>
     </dataValidation>
   </dataValidations>
@@ -8145,22 +8817,22 @@
     <mergeCell ref="A1:L1"/>
   </mergeCells>
   <dataValidations count="6">
-    <dataValidation sqref="C3:C12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C3:C12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"سيدان,SUV,هايس / ميني باص,كوستر,أتوبيس,جيب,أخرى"</formula1>
     </dataValidation>
-    <dataValidation sqref="E3:E12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E3:E12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"ملك,إيجار"</formula1>
     </dataValidation>
-    <dataValidation sqref="H3:H12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H3:H12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"مشوار,يوم,شهر"</formula1>
     </dataValidation>
-    <dataValidation sqref="I3:I12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I3:I12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"جنيه,يورو"</formula1>
     </dataValidation>
-    <dataValidation sqref="J3:J12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J3:J12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"علينا,على المؤجر,على السواق"</formula1>
     </dataValidation>
-    <dataValidation sqref="L3:L12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L3:L12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"ناقص,اتملى,محتاج مراجعة,مش محتاجينه"</formula1>
     </dataValidation>
   </dataValidations>
@@ -8407,7 +9079,11 @@
           <t>رقم ترخيص وزارة السياحة (لو موجود)</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>لا يوجد ترخيص وزارة سياحة حاليًا</t>
+        </is>
+      </c>
       <c r="D7" s="5" t="inlineStr"/>
       <c r="E7" s="5" t="inlineStr">
         <is>
@@ -8416,7 +9092,7 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>ناقص</t>
+          <t>اتملى</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
@@ -8658,7 +9334,11 @@
           <t>إيميل بتوصله إشعارات الحجوزات</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr"/>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>ده متاح معاك (محمد) — الإيميل لسه هيتحدد</t>
+        </is>
+      </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
           <t>bookings@…</t>
@@ -8671,7 +9351,7 @@
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>ناقص</t>
+          <t>محتاج مراجعة</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr"/>
@@ -8689,7 +9369,7 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>12 ساعة يوميًا (ناقص: من الساعة كام لكام)</t>
+          <t>24 ساعة يوميًا</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -8704,7 +9384,7 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>محتاج مراجعة</t>
+          <t>اتملى</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -8724,7 +9404,11 @@
           <t>لغات الرد على العملاء</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr"/>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>عربي، إنجليزي، روسي</t>
+        </is>
+      </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
           <t>عربي، إنجليزي، روسي</t>
@@ -8737,7 +9421,7 @@
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>ناقص</t>
+          <t>اتملى</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr"/>
@@ -8753,7 +9437,9 @@
           <t>سنة بداية الشغل</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr"/>
+      <c r="C17" s="7" t="n">
+        <v>2024</v>
+      </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
           <t>2015</t>
@@ -8766,7 +9452,7 @@
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>ناقص</t>
+          <t>اتملى</t>
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr">
@@ -8811,7 +9497,11 @@
           <t>قصة قصيرة عن الشركة (سطرين-تلاتة)</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr"/>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>we do our best to make you happy</t>
+        </is>
+      </c>
       <c r="D19" s="5" t="inlineStr"/>
       <c r="E19" s="5" t="inlineStr">
         <is>
@@ -8820,7 +9510,7 @@
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>ناقص</t>
+          <t>محتاج مراجعة</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
@@ -9160,7 +9850,7 @@
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="E3:E10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E3:E10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"ناقص,اتملى,محتاج مراجعة,مش محتاجينه"</formula1>
     </dataValidation>
   </dataValidations>
@@ -9248,14 +9938,36 @@
           <t>super-safari-adventure</t>
         </is>
       </c>
-      <c r="B3" s="83" t="inlineStr"/>
-      <c r="C3" s="83" t="inlineStr"/>
-      <c r="D3" s="83" t="inlineStr"/>
-      <c r="E3" s="83" t="inlineStr"/>
+      <c r="B3" s="83" t="n">
+        <v>600</v>
+      </c>
+      <c r="C3" s="83" t="inlineStr">
+        <is>
+          <t>احمد</t>
+        </is>
+      </c>
+      <c r="D3" s="83" t="n">
+        <v>500</v>
+      </c>
+      <c r="E3" s="83" t="n">
+        <v>50</v>
+      </c>
       <c r="F3" s="83" t="inlineStr"/>
-      <c r="G3" s="83" t="inlineStr"/>
-      <c r="H3" s="83" t="inlineStr"/>
-      <c r="I3" s="83" t="inlineStr"/>
+      <c r="G3" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
+      <c r="H3" s="83" t="inlineStr">
+        <is>
+          <t>احنا</t>
+        </is>
+      </c>
+      <c r="I3" s="83" t="inlineStr">
+        <is>
+          <t>جمل 100</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="82" t="inlineStr">
@@ -9263,14 +9975,34 @@
           <t>sunset-quad-bike</t>
         </is>
       </c>
-      <c r="B4" s="83" t="inlineStr"/>
-      <c r="C4" s="83" t="inlineStr"/>
+      <c r="B4" s="83" t="n">
+        <v>600</v>
+      </c>
+      <c r="C4" s="83" t="inlineStr">
+        <is>
+          <t>احمد</t>
+        </is>
+      </c>
       <c r="D4" s="83" t="inlineStr"/>
-      <c r="E4" s="83" t="inlineStr"/>
+      <c r="E4" s="83" t="n">
+        <v>50</v>
+      </c>
       <c r="F4" s="83" t="inlineStr"/>
-      <c r="G4" s="83" t="inlineStr"/>
-      <c r="H4" s="83" t="inlineStr"/>
-      <c r="I4" s="83" t="inlineStr"/>
+      <c r="G4" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
+      <c r="H4" s="83" t="inlineStr">
+        <is>
+          <t>احنا</t>
+        </is>
+      </c>
+      <c r="I4" s="83" t="inlineStr">
+        <is>
+          <t>جمل 100</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="82" t="inlineStr">
@@ -9278,14 +10010,36 @@
           <t>double-buggy-camel-ride</t>
         </is>
       </c>
-      <c r="B5" s="83" t="inlineStr"/>
-      <c r="C5" s="83" t="inlineStr"/>
-      <c r="D5" s="83" t="inlineStr"/>
-      <c r="E5" s="83" t="inlineStr"/>
+      <c r="B5" s="83" t="n">
+        <v>1100</v>
+      </c>
+      <c r="C5" s="83" t="inlineStr">
+        <is>
+          <t>احمد</t>
+        </is>
+      </c>
+      <c r="D5" s="83" t="n">
+        <v>500</v>
+      </c>
+      <c r="E5" s="83" t="n">
+        <v>50</v>
+      </c>
       <c r="F5" s="83" t="inlineStr"/>
-      <c r="G5" s="83" t="inlineStr"/>
-      <c r="H5" s="83" t="inlineStr"/>
-      <c r="I5" s="83" t="inlineStr"/>
+      <c r="G5" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
+      <c r="H5" s="83" t="inlineStr">
+        <is>
+          <t>احنا</t>
+        </is>
+      </c>
+      <c r="I5" s="83" t="inlineStr">
+        <is>
+          <t>جمل 100</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="82" t="inlineStr">
@@ -9293,14 +10047,38 @@
           <t>bedouin-dinner-camel-ride</t>
         </is>
       </c>
-      <c r="B6" s="83" t="inlineStr"/>
-      <c r="C6" s="83" t="inlineStr"/>
+      <c r="B6" s="83" t="inlineStr">
+        <is>
+          <t>500+100</t>
+        </is>
+      </c>
+      <c r="C6" s="83" t="inlineStr">
+        <is>
+          <t>احمد</t>
+        </is>
+      </c>
       <c r="D6" s="83" t="inlineStr"/>
-      <c r="E6" s="83" t="inlineStr"/>
+      <c r="E6" s="83" t="inlineStr">
+        <is>
+          <t>500+100</t>
+        </is>
+      </c>
       <c r="F6" s="83" t="inlineStr"/>
-      <c r="G6" s="83" t="inlineStr"/>
-      <c r="H6" s="83" t="inlineStr"/>
-      <c r="I6" s="83" t="inlineStr"/>
+      <c r="G6" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
+      <c r="H6" s="83" t="inlineStr">
+        <is>
+          <t>احنا</t>
+        </is>
+      </c>
+      <c r="I6" s="83" t="inlineStr">
+        <is>
+          <t>جمل 100</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="82" t="inlineStr">
@@ -9308,14 +10086,38 @@
           <t>dahab-colored-canyon</t>
         </is>
       </c>
-      <c r="B7" s="83" t="inlineStr"/>
-      <c r="C7" s="83" t="inlineStr"/>
-      <c r="D7" s="83" t="inlineStr"/>
-      <c r="E7" s="83" t="inlineStr"/>
+      <c r="B7" s="83" t="n">
+        <v>700</v>
+      </c>
+      <c r="C7" s="83" t="inlineStr">
+        <is>
+          <t>محمد</t>
+        </is>
+      </c>
+      <c r="D7" s="83" t="inlineStr">
+        <is>
+          <t>شامل</t>
+        </is>
+      </c>
+      <c r="E7" s="83" t="n">
+        <v>50</v>
+      </c>
       <c r="F7" s="83" t="inlineStr"/>
-      <c r="G7" s="83" t="inlineStr"/>
-      <c r="H7" s="83" t="inlineStr"/>
-      <c r="I7" s="83" t="inlineStr"/>
+      <c r="G7" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
+      <c r="H7" s="83" t="inlineStr">
+        <is>
+          <t>احنا</t>
+        </is>
+      </c>
+      <c r="I7" s="83" t="inlineStr">
+        <is>
+          <t>شامل جيب +متسكلات</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="82" t="inlineStr">
@@ -9323,14 +10125,36 @@
           <t>camel-horse-ride</t>
         </is>
       </c>
-      <c r="B8" s="83" t="inlineStr"/>
-      <c r="C8" s="83" t="inlineStr"/>
-      <c r="D8" s="83" t="inlineStr"/>
+      <c r="B8" s="83" t="n">
+        <v>1300</v>
+      </c>
+      <c r="C8" s="83" t="inlineStr">
+        <is>
+          <t>عبدون</t>
+        </is>
+      </c>
+      <c r="D8" s="83" t="inlineStr">
+        <is>
+          <t>لا يوجد</t>
+        </is>
+      </c>
       <c r="E8" s="83" t="inlineStr"/>
       <c r="F8" s="83" t="inlineStr"/>
-      <c r="G8" s="83" t="inlineStr"/>
-      <c r="H8" s="83" t="inlineStr"/>
-      <c r="I8" s="83" t="inlineStr"/>
+      <c r="G8" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
+      <c r="H8" s="83" t="inlineStr">
+        <is>
+          <t>احنا</t>
+        </is>
+      </c>
+      <c r="I8" s="83" t="inlineStr">
+        <is>
+          <t>شامل نقل</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="82" t="inlineStr">
@@ -9338,13 +10162,31 @@
           <t>ras-mohamed-white-island-boat</t>
         </is>
       </c>
-      <c r="B9" s="83" t="inlineStr"/>
-      <c r="C9" s="83" t="inlineStr"/>
-      <c r="D9" s="83" t="inlineStr"/>
+      <c r="B9" s="83" t="n">
+        <v>1300</v>
+      </c>
+      <c r="C9" s="83" t="inlineStr">
+        <is>
+          <t>محمد</t>
+        </is>
+      </c>
+      <c r="D9" s="83" t="inlineStr">
+        <is>
+          <t>شامل</t>
+        </is>
+      </c>
       <c r="E9" s="83" t="inlineStr"/>
       <c r="F9" s="83" t="inlineStr"/>
-      <c r="G9" s="83" t="inlineStr"/>
-      <c r="H9" s="83" t="inlineStr"/>
+      <c r="G9" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
+      <c r="H9" s="83" t="inlineStr">
+        <is>
+          <t>احنا</t>
+        </is>
+      </c>
       <c r="I9" s="83" t="inlineStr"/>
     </row>
     <row r="10">
@@ -9353,13 +10195,31 @@
           <t>evening-cruise</t>
         </is>
       </c>
-      <c r="B10" s="83" t="inlineStr"/>
-      <c r="C10" s="83" t="inlineStr"/>
-      <c r="D10" s="83" t="inlineStr"/>
+      <c r="B10" s="83" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C10" s="83" t="inlineStr">
+        <is>
+          <t>عادل</t>
+        </is>
+      </c>
+      <c r="D10" s="83" t="inlineStr">
+        <is>
+          <t>شامل</t>
+        </is>
+      </c>
       <c r="E10" s="83" t="inlineStr"/>
       <c r="F10" s="83" t="inlineStr"/>
-      <c r="G10" s="83" t="inlineStr"/>
-      <c r="H10" s="83" t="inlineStr"/>
+      <c r="G10" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
+      <c r="H10" s="83" t="inlineStr">
+        <is>
+          <t>احنا</t>
+        </is>
+      </c>
       <c r="I10" s="83" t="inlineStr"/>
     </row>
     <row r="11">
@@ -9368,14 +10228,32 @@
           <t>glass-bottom-boat</t>
         </is>
       </c>
-      <c r="B11" s="83" t="inlineStr"/>
-      <c r="C11" s="83" t="inlineStr"/>
+      <c r="B11" s="83" t="n">
+        <v>300</v>
+      </c>
+      <c r="C11" s="83" t="inlineStr">
+        <is>
+          <t>روماني</t>
+        </is>
+      </c>
       <c r="D11" s="83" t="inlineStr"/>
       <c r="E11" s="83" t="inlineStr"/>
       <c r="F11" s="83" t="inlineStr"/>
-      <c r="G11" s="83" t="inlineStr"/>
-      <c r="H11" s="83" t="inlineStr"/>
-      <c r="I11" s="83" t="inlineStr"/>
+      <c r="G11" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
+      <c r="H11" s="83" t="inlineStr">
+        <is>
+          <t>احنا</t>
+        </is>
+      </c>
+      <c r="I11" s="83" t="inlineStr">
+        <is>
+          <t>شامل نقل</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="82" t="inlineStr">
@@ -9383,14 +10261,32 @@
           <t>diving-course</t>
         </is>
       </c>
-      <c r="B12" s="83" t="inlineStr"/>
-      <c r="C12" s="83" t="inlineStr"/>
+      <c r="B12" s="83" t="n">
+        <v>17000</v>
+      </c>
+      <c r="C12" s="83" t="inlineStr">
+        <is>
+          <t>محمد</t>
+        </is>
+      </c>
       <c r="D12" s="83" t="inlineStr"/>
       <c r="E12" s="83" t="inlineStr"/>
       <c r="F12" s="83" t="inlineStr"/>
-      <c r="G12" s="83" t="inlineStr"/>
-      <c r="H12" s="83" t="inlineStr"/>
-      <c r="I12" s="83" t="inlineStr"/>
+      <c r="G12" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
+      <c r="H12" s="83" t="inlineStr">
+        <is>
+          <t>احنا</t>
+        </is>
+      </c>
+      <c r="I12" s="83" t="inlineStr">
+        <is>
+          <t>شامل نقل</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="82" t="inlineStr">
@@ -9398,13 +10294,27 @@
           <t>sinai-dream-sailboat</t>
         </is>
       </c>
-      <c r="B13" s="83" t="inlineStr"/>
+      <c r="B13" s="83" t="n">
+        <v>3250</v>
+      </c>
       <c r="C13" s="83" t="inlineStr"/>
-      <c r="D13" s="83" t="inlineStr"/>
+      <c r="D13" s="83" t="inlineStr">
+        <is>
+          <t>شامل</t>
+        </is>
+      </c>
       <c r="E13" s="83" t="inlineStr"/>
       <c r="F13" s="83" t="inlineStr"/>
-      <c r="G13" s="83" t="inlineStr"/>
-      <c r="H13" s="83" t="inlineStr"/>
+      <c r="G13" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
+      <c r="H13" s="83" t="inlineStr">
+        <is>
+          <t>احنا</t>
+        </is>
+      </c>
       <c r="I13" s="83" t="inlineStr"/>
     </row>
     <row r="14">
@@ -9413,14 +10323,32 @@
           <t>ras-mohamed-by-bus</t>
         </is>
       </c>
-      <c r="B14" s="83" t="inlineStr"/>
+      <c r="B14" s="83" t="n">
+        <v>700</v>
+      </c>
       <c r="C14" s="83" t="inlineStr"/>
-      <c r="D14" s="83" t="inlineStr"/>
+      <c r="D14" s="83" t="inlineStr">
+        <is>
+          <t>لا يوجد</t>
+        </is>
+      </c>
       <c r="E14" s="83" t="inlineStr"/>
       <c r="F14" s="83" t="inlineStr"/>
-      <c r="G14" s="83" t="inlineStr"/>
-      <c r="H14" s="83" t="inlineStr"/>
-      <c r="I14" s="83" t="inlineStr"/>
+      <c r="G14" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
+      <c r="H14" s="83" t="inlineStr">
+        <is>
+          <t>احنا</t>
+        </is>
+      </c>
+      <c r="I14" s="83" t="inlineStr">
+        <is>
+          <t>شامل نقل</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="82" t="inlineStr">
@@ -9428,14 +10356,32 @@
           <t>banana-boat</t>
         </is>
       </c>
-      <c r="B15" s="83" t="inlineStr"/>
+      <c r="B15" s="83" t="n">
+        <v>700</v>
+      </c>
       <c r="C15" s="83" t="inlineStr"/>
-      <c r="D15" s="83" t="inlineStr"/>
+      <c r="D15" s="83" t="inlineStr">
+        <is>
+          <t>لا يوجد</t>
+        </is>
+      </c>
       <c r="E15" s="83" t="inlineStr"/>
       <c r="F15" s="83" t="inlineStr"/>
-      <c r="G15" s="83" t="inlineStr"/>
-      <c r="H15" s="83" t="inlineStr"/>
-      <c r="I15" s="83" t="inlineStr"/>
+      <c r="G15" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
+      <c r="H15" s="83" t="inlineStr">
+        <is>
+          <t>احنا</t>
+        </is>
+      </c>
+      <c r="I15" s="83" t="inlineStr">
+        <is>
+          <t>شامل نقل</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="82" t="inlineStr">
@@ -9443,14 +10389,34 @@
           <t>parasailing-adventure</t>
         </is>
       </c>
-      <c r="B16" s="83" t="inlineStr"/>
+      <c r="B16" s="83" t="inlineStr">
+        <is>
+          <t>600/800</t>
+        </is>
+      </c>
       <c r="C16" s="83" t="inlineStr"/>
-      <c r="D16" s="83" t="inlineStr"/>
+      <c r="D16" s="83" t="inlineStr">
+        <is>
+          <t>لا يوجد</t>
+        </is>
+      </c>
       <c r="E16" s="83" t="inlineStr"/>
       <c r="F16" s="83" t="inlineStr"/>
-      <c r="G16" s="83" t="inlineStr"/>
-      <c r="H16" s="83" t="inlineStr"/>
-      <c r="I16" s="83" t="inlineStr"/>
+      <c r="G16" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
+      <c r="H16" s="83" t="inlineStr">
+        <is>
+          <t>احنا</t>
+        </is>
+      </c>
+      <c r="I16" s="83" t="inlineStr">
+        <is>
+          <t>شامل نقل</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="82" t="inlineStr">
@@ -9458,14 +10424,32 @@
           <t>speed-boat-adventure</t>
         </is>
       </c>
-      <c r="B17" s="83" t="inlineStr"/>
+      <c r="B17" s="83" t="n">
+        <v>4200</v>
+      </c>
       <c r="C17" s="83" t="inlineStr"/>
-      <c r="D17" s="83" t="inlineStr"/>
+      <c r="D17" s="83" t="inlineStr">
+        <is>
+          <t>حسب الطلب</t>
+        </is>
+      </c>
       <c r="E17" s="83" t="inlineStr"/>
       <c r="F17" s="83" t="inlineStr"/>
-      <c r="G17" s="83" t="inlineStr"/>
-      <c r="H17" s="83" t="inlineStr"/>
-      <c r="I17" s="83" t="inlineStr"/>
+      <c r="G17" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
+      <c r="H17" s="83" t="inlineStr">
+        <is>
+          <t>احنا</t>
+        </is>
+      </c>
+      <c r="I17" s="83" t="inlineStr">
+        <is>
+          <t>شامل نقل</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="82" t="inlineStr">
@@ -9473,14 +10457,32 @@
           <t>submarine</t>
         </is>
       </c>
-      <c r="B18" s="83" t="inlineStr"/>
+      <c r="B18" s="83" t="n">
+        <v>1400</v>
+      </c>
       <c r="C18" s="83" t="inlineStr"/>
-      <c r="D18" s="83" t="inlineStr"/>
+      <c r="D18" s="83" t="inlineStr">
+        <is>
+          <t>لا يوجد</t>
+        </is>
+      </c>
       <c r="E18" s="83" t="inlineStr"/>
       <c r="F18" s="83" t="inlineStr"/>
-      <c r="G18" s="83" t="inlineStr"/>
-      <c r="H18" s="83" t="inlineStr"/>
-      <c r="I18" s="83" t="inlineStr"/>
+      <c r="G18" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
+      <c r="H18" s="83" t="inlineStr">
+        <is>
+          <t>احنا</t>
+        </is>
+      </c>
+      <c r="I18" s="83" t="inlineStr">
+        <is>
+          <t>شامل نقل</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="82" t="inlineStr">
@@ -9488,13 +10490,27 @@
           <t>tiran-island-boat-trip</t>
         </is>
       </c>
-      <c r="B19" s="83" t="inlineStr"/>
+      <c r="B19" s="83" t="n">
+        <v>1300</v>
+      </c>
       <c r="C19" s="83" t="inlineStr"/>
-      <c r="D19" s="83" t="inlineStr"/>
+      <c r="D19" s="83" t="inlineStr">
+        <is>
+          <t>شامل</t>
+        </is>
+      </c>
       <c r="E19" s="83" t="inlineStr"/>
       <c r="F19" s="83" t="inlineStr"/>
-      <c r="G19" s="83" t="inlineStr"/>
-      <c r="H19" s="83" t="inlineStr"/>
+      <c r="G19" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
+      <c r="H19" s="83" t="inlineStr">
+        <is>
+          <t>احنا</t>
+        </is>
+      </c>
       <c r="I19" s="83" t="inlineStr"/>
     </row>
     <row r="20">
@@ -9503,13 +10519,27 @@
           <t>tube-boat</t>
         </is>
       </c>
-      <c r="B20" s="83" t="inlineStr"/>
+      <c r="B20" s="83" t="n">
+        <v>700</v>
+      </c>
       <c r="C20" s="83" t="inlineStr"/>
-      <c r="D20" s="83" t="inlineStr"/>
+      <c r="D20" s="83" t="inlineStr">
+        <is>
+          <t>شامل</t>
+        </is>
+      </c>
       <c r="E20" s="83" t="inlineStr"/>
       <c r="F20" s="83" t="inlineStr"/>
-      <c r="G20" s="83" t="inlineStr"/>
-      <c r="H20" s="83" t="inlineStr"/>
+      <c r="G20" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
+      <c r="H20" s="83" t="inlineStr">
+        <is>
+          <t>احنا</t>
+        </is>
+      </c>
       <c r="I20" s="83" t="inlineStr"/>
     </row>
     <row r="21">
@@ -9518,13 +10548,27 @@
           <t>cairo-by-bus</t>
         </is>
       </c>
-      <c r="B21" s="83" t="inlineStr"/>
+      <c r="B21" s="83" t="n">
+        <v>1900</v>
+      </c>
       <c r="C21" s="83" t="inlineStr"/>
-      <c r="D21" s="83" t="inlineStr"/>
+      <c r="D21" s="83" t="inlineStr">
+        <is>
+          <t>شامل</t>
+        </is>
+      </c>
       <c r="E21" s="83" t="inlineStr"/>
       <c r="F21" s="83" t="inlineStr"/>
-      <c r="G21" s="83" t="inlineStr"/>
-      <c r="H21" s="83" t="inlineStr"/>
+      <c r="G21" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
+      <c r="H21" s="83" t="inlineStr">
+        <is>
+          <t>احنا</t>
+        </is>
+      </c>
       <c r="I21" s="83" t="inlineStr"/>
     </row>
     <row r="22">
@@ -9533,13 +10577,27 @@
           <t>cairo-by-plane</t>
         </is>
       </c>
-      <c r="B22" s="83" t="inlineStr"/>
+      <c r="B22" s="83" t="n">
+        <v>12000</v>
+      </c>
       <c r="C22" s="83" t="inlineStr"/>
-      <c r="D22" s="83" t="inlineStr"/>
+      <c r="D22" s="83" t="inlineStr">
+        <is>
+          <t>شامل</t>
+        </is>
+      </c>
       <c r="E22" s="83" t="inlineStr"/>
       <c r="F22" s="83" t="inlineStr"/>
-      <c r="G22" s="83" t="inlineStr"/>
-      <c r="H22" s="83" t="inlineStr"/>
+      <c r="G22" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
+      <c r="H22" s="83" t="inlineStr">
+        <is>
+          <t>احنا</t>
+        </is>
+      </c>
       <c r="I22" s="83" t="inlineStr"/>
     </row>
     <row r="23">
@@ -9548,13 +10606,27 @@
           <t>mount-sinai-st-catherine</t>
         </is>
       </c>
-      <c r="B23" s="83" t="inlineStr"/>
+      <c r="B23" s="83" t="n">
+        <v>1400</v>
+      </c>
       <c r="C23" s="83" t="inlineStr"/>
-      <c r="D23" s="83" t="inlineStr"/>
+      <c r="D23" s="83" t="inlineStr">
+        <is>
+          <t>لا يوجد</t>
+        </is>
+      </c>
       <c r="E23" s="83" t="inlineStr"/>
       <c r="F23" s="83" t="inlineStr"/>
-      <c r="G23" s="83" t="inlineStr"/>
-      <c r="H23" s="83" t="inlineStr"/>
+      <c r="G23" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
+      <c r="H23" s="83" t="inlineStr">
+        <is>
+          <t>احنا</t>
+        </is>
+      </c>
       <c r="I23" s="83" t="inlineStr"/>
     </row>
     <row r="24">
@@ -9563,13 +10635,27 @@
           <t>luxor-by-plane</t>
         </is>
       </c>
-      <c r="B24" s="83" t="inlineStr"/>
+      <c r="B24" s="83" t="n">
+        <v>12500</v>
+      </c>
       <c r="C24" s="83" t="inlineStr"/>
-      <c r="D24" s="83" t="inlineStr"/>
+      <c r="D24" s="83" t="inlineStr">
+        <is>
+          <t>شامل</t>
+        </is>
+      </c>
       <c r="E24" s="83" t="inlineStr"/>
       <c r="F24" s="83" t="inlineStr"/>
-      <c r="G24" s="83" t="inlineStr"/>
-      <c r="H24" s="83" t="inlineStr"/>
+      <c r="G24" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
+      <c r="H24" s="83" t="inlineStr">
+        <is>
+          <t>احنا</t>
+        </is>
+      </c>
       <c r="I24" s="83" t="inlineStr"/>
     </row>
     <row r="25">
@@ -9578,13 +10664,27 @@
           <t>st-catherine-dahab</t>
         </is>
       </c>
-      <c r="B25" s="83" t="inlineStr"/>
+      <c r="B25" s="83" t="n">
+        <v>1400</v>
+      </c>
       <c r="C25" s="83" t="inlineStr"/>
-      <c r="D25" s="83" t="inlineStr"/>
+      <c r="D25" s="83" t="inlineStr">
+        <is>
+          <t>شامل</t>
+        </is>
+      </c>
       <c r="E25" s="83" t="inlineStr"/>
       <c r="F25" s="83" t="inlineStr"/>
-      <c r="G25" s="83" t="inlineStr"/>
-      <c r="H25" s="83" t="inlineStr"/>
+      <c r="G25" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
+      <c r="H25" s="83" t="inlineStr">
+        <is>
+          <t>احنا</t>
+        </is>
+      </c>
       <c r="I25" s="83" t="inlineStr"/>
     </row>
     <row r="26">
@@ -9593,14 +10693,28 @@
           <t>turkish-bath</t>
         </is>
       </c>
-      <c r="B26" s="83" t="inlineStr"/>
+      <c r="B26" s="83" t="n">
+        <v>1300</v>
+      </c>
       <c r="C26" s="83" t="inlineStr"/>
       <c r="D26" s="83" t="inlineStr"/>
       <c r="E26" s="83" t="inlineStr"/>
       <c r="F26" s="83" t="inlineStr"/>
-      <c r="G26" s="83" t="inlineStr"/>
-      <c r="H26" s="83" t="inlineStr"/>
-      <c r="I26" s="83" t="inlineStr"/>
+      <c r="G26" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
+      <c r="H26" s="83" t="inlineStr">
+        <is>
+          <t>احنا</t>
+        </is>
+      </c>
+      <c r="I26" s="83" t="inlineStr">
+        <is>
+          <t>شامل نقل</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="82" t="inlineStr">
@@ -9608,14 +10722,28 @@
           <t>dolphin-show</t>
         </is>
       </c>
-      <c r="B27" s="83" t="inlineStr"/>
+      <c r="B27" s="83" t="n">
+        <v>650</v>
+      </c>
       <c r="C27" s="83" t="inlineStr"/>
       <c r="D27" s="83" t="inlineStr"/>
       <c r="E27" s="83" t="inlineStr"/>
       <c r="F27" s="83" t="inlineStr"/>
-      <c r="G27" s="83" t="inlineStr"/>
-      <c r="H27" s="83" t="inlineStr"/>
-      <c r="I27" s="83" t="inlineStr"/>
+      <c r="G27" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
+      <c r="H27" s="83" t="inlineStr">
+        <is>
+          <t>احنا</t>
+        </is>
+      </c>
+      <c r="I27" s="83" t="inlineStr">
+        <is>
+          <t>شامل نقل</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="82" t="inlineStr">
@@ -9623,14 +10751,28 @@
           <t>swimming-with-dolphins</t>
         </is>
       </c>
-      <c r="B28" s="83" t="inlineStr"/>
+      <c r="B28" s="83" t="n">
+        <v>3500</v>
+      </c>
       <c r="C28" s="83" t="inlineStr"/>
       <c r="D28" s="83" t="inlineStr"/>
       <c r="E28" s="83" t="inlineStr"/>
       <c r="F28" s="83" t="inlineStr"/>
-      <c r="G28" s="83" t="inlineStr"/>
-      <c r="H28" s="83" t="inlineStr"/>
-      <c r="I28" s="83" t="inlineStr"/>
+      <c r="G28" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
+      <c r="H28" s="83" t="inlineStr">
+        <is>
+          <t>احنا</t>
+        </is>
+      </c>
+      <c r="I28" s="83" t="inlineStr">
+        <is>
+          <t>شامل نقل</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="82" t="inlineStr">
@@ -9638,24 +10780,38 @@
           <t>sharm-airport-transfer</t>
         </is>
       </c>
-      <c r="B29" s="83" t="inlineStr"/>
+      <c r="B29" s="83" t="n">
+        <v>600</v>
+      </c>
       <c r="C29" s="83" t="inlineStr"/>
       <c r="D29" s="83" t="inlineStr"/>
       <c r="E29" s="83" t="inlineStr"/>
       <c r="F29" s="83" t="inlineStr"/>
-      <c r="G29" s="83" t="inlineStr"/>
-      <c r="H29" s="83" t="inlineStr"/>
-      <c r="I29" s="83" t="inlineStr"/>
+      <c r="G29" s="83" t="inlineStr">
+        <is>
+          <t>جنيه</t>
+        </is>
+      </c>
+      <c r="H29" s="83" t="inlineStr">
+        <is>
+          <t>احنا</t>
+        </is>
+      </c>
+      <c r="I29" s="83" t="inlineStr">
+        <is>
+          <t>شامل نقل</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="G3:G29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G3:G29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"جنيه,يورو"</formula1>
     </dataValidation>
-    <dataValidation sqref="H3:H29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H3:H29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"احنا,المورد,العميل"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
docs(safari-owner-data): fill settlement, commission, refund and cash-box defaults under owner delegation (marked for review)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/clients/safari-tours-sharm/owner-data/safari-tours-owner-data-hub.xlsx
+++ b/clients/safari-tours-sharm/owner-data/safari-tours-owner-data-hub.xlsx
@@ -126,7 +126,7 @@
       <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -193,6 +193,11 @@
         <fgColor rgb="00E2F0D9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCE4D6"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="7">
     <border/>
@@ -245,7 +250,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="85">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -467,6 +472,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1564,7 +1572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1756,6 +1764,23 @@
       <c r="C11" t="inlineStr">
         <is>
           <t>دمج ملف محمد «safari-tours-owner-data (1).xlsx»: 5 موردين، أسعار الموردين لكل الرحلات، 4 سواقين، تكاليف الرحلات، وبيانات الشركة (ساعات الدعم 24 ساعة، اللغات، سنة البداية، مفيش ترخيص سياحة حاليًا). العربيات فاضية لحد ما تتوفر البيانات.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ملأ قواعد التسويات والعمولات ورد الفلوس والخزنة بافتراضات معقولة بتفويض محمد («لو في نواقص املاها ولما نرجع أعدّل»). كلها معلّمة «محتاج مراجعة».</t>
         </is>
       </c>
     </row>
@@ -7172,7 +7197,11 @@
         <v>46032</v>
       </c>
       <c r="J3" s="83" t="inlineStr"/>
-      <c r="K3" s="83" t="inlineStr"/>
+      <c r="K3" s="83" t="inlineStr">
+        <is>
+          <t>السعر ده بيتعامل كسعر الرحلة عند أي مورد بيشغّلها لحد ما يتحدد المورد (افتراض Claude 2026-10-07 — عدّله لو مختلف)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="82" t="inlineStr">
@@ -7205,7 +7234,11 @@
         <v>46032</v>
       </c>
       <c r="J4" s="83" t="inlineStr"/>
-      <c r="K4" s="83" t="inlineStr"/>
+      <c r="K4" s="83" t="inlineStr">
+        <is>
+          <t>السعر ده بيتعامل كسعر الرحلة عند أي مورد بيشغّلها لحد ما يتحدد المورد (افتراض Claude 2026-10-07 — عدّله لو مختلف)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="82" t="inlineStr">
@@ -7238,7 +7271,11 @@
         <v>46032</v>
       </c>
       <c r="J5" s="83" t="inlineStr"/>
-      <c r="K5" s="83" t="inlineStr"/>
+      <c r="K5" s="83" t="inlineStr">
+        <is>
+          <t>السعر ده بيتعامل كسعر الرحلة عند أي مورد بيشغّلها لحد ما يتحدد المورد (افتراض Claude 2026-10-07 — عدّله لو مختلف)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="82" t="inlineStr">
@@ -7271,7 +7308,11 @@
         <v>46032</v>
       </c>
       <c r="J6" s="83" t="inlineStr"/>
-      <c r="K6" s="83" t="inlineStr"/>
+      <c r="K6" s="83" t="inlineStr">
+        <is>
+          <t>السعر ده بيتعامل كسعر الرحلة عند أي مورد بيشغّلها لحد ما يتحدد المورد (افتراض Claude 2026-10-07 — عدّله لو مختلف)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="82" t="inlineStr">
@@ -7306,7 +7347,7 @@
       <c r="J7" s="83" t="inlineStr"/>
       <c r="K7" s="83" t="inlineStr">
         <is>
-          <t>جيب +جمل +بتش بجي</t>
+          <t>جيب +جمل +بتش بجي | السعر ده بيتعامل كسعر الرحلة عند أي مورد بيشغّلها لحد ما يتحدد المورد (افتراض Claude 2026-10-07 — عدّله لو مختلف)</t>
         </is>
       </c>
     </row>
@@ -7341,7 +7382,11 @@
         <v>46305</v>
       </c>
       <c r="J8" s="83" t="inlineStr"/>
-      <c r="K8" s="83" t="inlineStr"/>
+      <c r="K8" s="83" t="inlineStr">
+        <is>
+          <t>السعر ده بيتعامل كسعر الرحلة عند أي مورد بيشغّلها لحد ما يتحدد المورد (افتراض Claude 2026-10-07 — عدّله لو مختلف)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="82" t="inlineStr">
@@ -7376,7 +7421,7 @@
       <c r="J9" s="83" t="inlineStr"/>
       <c r="K9" s="83" t="inlineStr">
         <is>
-          <t>غداء سوفت درينك</t>
+          <t>غداء سوفت درينك | السعر ده بيتعامل كسعر الرحلة عند أي مورد بيشغّلها لحد ما يتحدد المورد (افتراض Claude 2026-10-07 — عدّله لو مختلف)</t>
         </is>
       </c>
     </row>
@@ -7411,7 +7456,11 @@
         <v>46032</v>
       </c>
       <c r="J10" s="83" t="inlineStr"/>
-      <c r="K10" s="83" t="inlineStr"/>
+      <c r="K10" s="83" t="inlineStr">
+        <is>
+          <t>السعر ده بيتعامل كسعر الرحلة عند أي مورد بيشغّلها لحد ما يتحدد المورد (افتراض Claude 2026-10-07 — عدّله لو مختلف)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="82" t="inlineStr">
@@ -7444,7 +7493,11 @@
         <v>46031</v>
       </c>
       <c r="J11" s="83" t="inlineStr"/>
-      <c r="K11" s="83" t="inlineStr"/>
+      <c r="K11" s="83" t="inlineStr">
+        <is>
+          <t>السعر ده بيتعامل كسعر الرحلة عند أي مورد بيشغّلها لحد ما يتحدد المورد (افتراض Claude 2026-10-07 — عدّله لو مختلف)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="82" t="inlineStr">
@@ -7477,7 +7530,11 @@
         <v>46028</v>
       </c>
       <c r="J12" s="83" t="inlineStr"/>
-      <c r="K12" s="83" t="inlineStr"/>
+      <c r="K12" s="83" t="inlineStr">
+        <is>
+          <t>السعر ده بيتعامل كسعر الرحلة عند أي مورد بيشغّلها لحد ما يتحدد المورد (افتراض Claude 2026-10-07 — عدّله لو مختلف)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="82" t="inlineStr">
@@ -7510,7 +7567,11 @@
         <v>46028</v>
       </c>
       <c r="J13" s="83" t="inlineStr"/>
-      <c r="K13" s="83" t="inlineStr"/>
+      <c r="K13" s="83" t="inlineStr">
+        <is>
+          <t>السعر ده بيتعامل كسعر الرحلة عند أي مورد بيشغّلها لحد ما يتحدد المورد (افتراض Claude 2026-10-07 — عدّله لو مختلف)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="82" t="inlineStr">
@@ -7543,7 +7604,11 @@
         <v>46023</v>
       </c>
       <c r="J14" s="83" t="inlineStr"/>
-      <c r="K14" s="83" t="inlineStr"/>
+      <c r="K14" s="83" t="inlineStr">
+        <is>
+          <t>السعر ده بيتعامل كسعر الرحلة عند أي مورد بيشغّلها لحد ما يتحدد المورد (افتراض Claude 2026-10-07 — عدّله لو مختلف)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="82" t="inlineStr">
@@ -7576,7 +7641,11 @@
         <v>46209</v>
       </c>
       <c r="J15" s="83" t="inlineStr"/>
-      <c r="K15" s="83" t="inlineStr"/>
+      <c r="K15" s="83" t="inlineStr">
+        <is>
+          <t>السعر ده بيتعامل كسعر الرحلة عند أي مورد بيشغّلها لحد ما يتحدد المورد (افتراض Claude 2026-10-07 — عدّله لو مختلف)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="82" t="inlineStr">
@@ -7613,7 +7682,7 @@
       <c r="J16" s="83" t="inlineStr"/>
       <c r="K16" s="83" t="inlineStr">
         <is>
-          <t>snigel 600 doubel 800</t>
+          <t>snigel 600 doubel 800 | السعر ده بيتعامل كسعر الرحلة عند أي مورد بيشغّلها لحد ما يتحدد المورد (افتراض Claude 2026-10-07 — عدّله لو مختلف)</t>
         </is>
       </c>
     </row>
@@ -7650,7 +7719,7 @@
       <c r="J17" s="83" t="inlineStr"/>
       <c r="K17" s="83" t="inlineStr">
         <is>
-          <t>سعر الساعه 5000</t>
+          <t>سعر الساعه 5000 | السعر ده بيتعامل كسعر الرحلة عند أي مورد بيشغّلها لحد ما يتحدد المورد (افتراض Claude 2026-10-07 — عدّله لو مختلف)</t>
         </is>
       </c>
     </row>
@@ -7685,7 +7754,11 @@
         <v>46028</v>
       </c>
       <c r="J18" s="83" t="inlineStr"/>
-      <c r="K18" s="83" t="inlineStr"/>
+      <c r="K18" s="83" t="inlineStr">
+        <is>
+          <t>السعر ده بيتعامل كسعر الرحلة عند أي مورد بيشغّلها لحد ما يتحدد المورد (افتراض Claude 2026-10-07 — عدّله لو مختلف)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="82" t="inlineStr">
@@ -7720,7 +7793,7 @@
       <c r="J19" s="83" t="inlineStr"/>
       <c r="K19" s="83" t="inlineStr">
         <is>
-          <t>غداء سوفت درينك</t>
+          <t>غداء سوفت درينك | السعر ده بيتعامل كسعر الرحلة عند أي مورد بيشغّلها لحد ما يتحدد المورد (افتراض Claude 2026-10-07 — عدّله لو مختلف)</t>
         </is>
       </c>
     </row>
@@ -7755,7 +7828,11 @@
         <v>46027</v>
       </c>
       <c r="J20" s="83" t="inlineStr"/>
-      <c r="K20" s="83" t="inlineStr"/>
+      <c r="K20" s="83" t="inlineStr">
+        <is>
+          <t>السعر ده بيتعامل كسعر الرحلة عند أي مورد بيشغّلها لحد ما يتحدد المورد (افتراض Claude 2026-10-07 — عدّله لو مختلف)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="82" t="inlineStr">
@@ -7788,7 +7865,11 @@
         <v>46023</v>
       </c>
       <c r="J21" s="83" t="inlineStr"/>
-      <c r="K21" s="83" t="inlineStr"/>
+      <c r="K21" s="83" t="inlineStr">
+        <is>
+          <t>السعر ده بيتعامل كسعر الرحلة عند أي مورد بيشغّلها لحد ما يتحدد المورد (افتراض Claude 2026-10-07 — عدّله لو مختلف)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="82" t="inlineStr">
@@ -7821,7 +7902,11 @@
         <v>46023</v>
       </c>
       <c r="J22" s="83" t="inlineStr"/>
-      <c r="K22" s="83" t="inlineStr"/>
+      <c r="K22" s="83" t="inlineStr">
+        <is>
+          <t>السعر ده بيتعامل كسعر الرحلة عند أي مورد بيشغّلها لحد ما يتحدد المورد (افتراض Claude 2026-10-07 — عدّله لو مختلف)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="82" t="inlineStr">
@@ -7854,7 +7939,11 @@
         <v>46023</v>
       </c>
       <c r="J23" s="83" t="inlineStr"/>
-      <c r="K23" s="83" t="inlineStr"/>
+      <c r="K23" s="83" t="inlineStr">
+        <is>
+          <t>السعر ده بيتعامل كسعر الرحلة عند أي مورد بيشغّلها لحد ما يتحدد المورد (افتراض Claude 2026-10-07 — عدّله لو مختلف)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="82" t="inlineStr">
@@ -7887,7 +7976,11 @@
         <v>46023</v>
       </c>
       <c r="J24" s="83" t="inlineStr"/>
-      <c r="K24" s="83" t="inlineStr"/>
+      <c r="K24" s="83" t="inlineStr">
+        <is>
+          <t>السعر ده بيتعامل كسعر الرحلة عند أي مورد بيشغّلها لحد ما يتحدد المورد (افتراض Claude 2026-10-07 — عدّله لو مختلف)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="82" t="inlineStr">
@@ -7920,7 +8013,11 @@
         <v>46023</v>
       </c>
       <c r="J25" s="83" t="inlineStr"/>
-      <c r="K25" s="83" t="inlineStr"/>
+      <c r="K25" s="83" t="inlineStr">
+        <is>
+          <t>السعر ده بيتعامل كسعر الرحلة عند أي مورد بيشغّلها لحد ما يتحدد المورد (افتراض Claude 2026-10-07 — عدّله لو مختلف)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="82" t="inlineStr">
@@ -7953,7 +8050,11 @@
         <v>46023</v>
       </c>
       <c r="J26" s="83" t="inlineStr"/>
-      <c r="K26" s="83" t="inlineStr"/>
+      <c r="K26" s="83" t="inlineStr">
+        <is>
+          <t>السعر ده بيتعامل كسعر الرحلة عند أي مورد بيشغّلها لحد ما يتحدد المورد (افتراض Claude 2026-10-07 — عدّله لو مختلف)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="82" t="inlineStr">
@@ -7986,7 +8087,11 @@
         <v>46023</v>
       </c>
       <c r="J27" s="83" t="inlineStr"/>
-      <c r="K27" s="83" t="inlineStr"/>
+      <c r="K27" s="83" t="inlineStr">
+        <is>
+          <t>السعر ده بيتعامل كسعر الرحلة عند أي مورد بيشغّلها لحد ما يتحدد المورد (افتراض Claude 2026-10-07 — عدّله لو مختلف)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="82" t="inlineStr">
@@ -8019,7 +8124,11 @@
         <v>46023</v>
       </c>
       <c r="J28" s="83" t="inlineStr"/>
-      <c r="K28" s="83" t="inlineStr"/>
+      <c r="K28" s="83" t="inlineStr">
+        <is>
+          <t>السعر ده بيتعامل كسعر الرحلة عند أي مورد بيشغّلها لحد ما يتحدد المورد (افتراض Claude 2026-10-07 — عدّله لو مختلف)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="82" t="inlineStr">
@@ -8052,7 +8161,11 @@
         <v>46023</v>
       </c>
       <c r="J29" s="83" t="inlineStr"/>
-      <c r="K29" s="83" t="inlineStr"/>
+      <c r="K29" s="83" t="inlineStr">
+        <is>
+          <t>السعر ده بيتعامل كسعر الرحلة عند أي مورد بيشغّلها لحد ما يتحدد المورد (افتراض Claude 2026-10-07 — عدّله لو مختلف)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -9672,7 +9785,11 @@
           <t>مين يعتمد الدفع للمورد أو السواق؟</t>
         </is>
       </c>
-      <c r="C3" s="83" t="inlineStr"/>
+      <c r="C3" s="85" t="inlineStr">
+        <is>
+          <t>محمد يعتمد أي دفع للمورد أو السواق (افتراض Claude 2026-10-07 — عدّله لو مختلف)</t>
+        </is>
+      </c>
       <c r="D3" s="82" t="inlineStr">
         <is>
           <t>محمد بس / محمد أو المدير</t>
@@ -9680,7 +9797,7 @@
       </c>
       <c r="E3" s="82" t="inlineStr">
         <is>
-          <t>ناقص</t>
+          <t>محتاج مراجعة</t>
         </is>
       </c>
     </row>
@@ -9695,7 +9812,11 @@
           <t>فيه مبلغ يقدر المدير يدفعه من غير اعتمادك؟ كام؟</t>
         </is>
       </c>
-      <c r="C4" s="83" t="inlineStr"/>
+      <c r="C4" s="85" t="inlineStr">
+        <is>
+          <t>المدير يدفع لحد 5000 جنيه للمورد/السواق في المرة من غير اعتماد محمد؛ أكتر من كده لازم محمد (افتراض Claude 2026-10-07 — عدّله لو مختلف)</t>
+        </is>
+      </c>
       <c r="D4" s="82" t="inlineStr">
         <is>
           <t>لحد 5000 جنيه</t>
@@ -9703,7 +9824,7 @@
       </c>
       <c r="E4" s="82" t="inlineStr">
         <is>
-          <t>ناقص</t>
+          <t>محتاج مراجعة</t>
         </is>
       </c>
     </row>
@@ -9718,7 +9839,11 @@
           <t>الحساب مع الموردين بالجنيه بيتحسب بنفس سعر اليوم اللي المدير بيحدده؟</t>
         </is>
       </c>
-      <c r="C5" s="83" t="inlineStr"/>
+      <c r="C5" s="85" t="inlineStr">
+        <is>
+          <t>الحساب مع الموردين والسواقين بالجنيه؛ لو احتجنا يورو نستخدم سعر اليوم اللي المدير بيحدده (افتراض Claude 2026-10-07 — عدّله لو مختلف)</t>
+        </is>
+      </c>
       <c r="D5" s="82" t="inlineStr">
         <is>
           <t>آه / لأ، بسعر متفق عليه</t>
@@ -9726,7 +9851,7 @@
       </c>
       <c r="E5" s="82" t="inlineStr">
         <is>
-          <t>ناقص</t>
+          <t>محتاج مراجعة</t>
         </is>
       </c>
     </row>
@@ -9741,7 +9866,11 @@
           <t>فيه عمولة لموظف المبيعات؟ كام ولمين؟</t>
         </is>
       </c>
-      <c r="C6" s="83" t="inlineStr"/>
+      <c r="C6" s="85" t="inlineStr">
+        <is>
+          <t>مفيش عمولة لموظف المبيعات حاليًا (افتراض Claude 2026-10-07 — عدّله لو مختلف)</t>
+        </is>
+      </c>
       <c r="D6" s="82" t="inlineStr">
         <is>
           <t>5% من البيع للي جاب العميل</t>
@@ -9749,7 +9878,7 @@
       </c>
       <c r="E6" s="82" t="inlineStr">
         <is>
-          <t>ناقص</t>
+          <t>محتاج مراجعة</t>
         </is>
       </c>
     </row>
@@ -9764,7 +9893,11 @@
           <t>فيه عمولة لفندق أو ريسبشن بيجيب عملاء؟ كام؟</t>
         </is>
       </c>
-      <c r="C7" s="83" t="inlineStr"/>
+      <c r="C7" s="85" t="inlineStr">
+        <is>
+          <t>مفيش عمولة لفندق أو ريسبشن حاليًا (السيستم يقدر يضيفها بنسبة أو مبلغ للفرد) (افتراض Claude 2026-10-07 — عدّله لو مختلف)</t>
+        </is>
+      </c>
       <c r="D7" s="82" t="inlineStr">
         <is>
           <t>10 يورو للفرد / 10%</t>
@@ -9772,7 +9905,7 @@
       </c>
       <c r="E7" s="82" t="inlineStr">
         <is>
-          <t>ناقص</t>
+          <t>محتاج مراجعة</t>
         </is>
       </c>
     </row>
@@ -9787,7 +9920,11 @@
           <t>العمولات بتتدفع إمتى وإزاي؟</t>
         </is>
       </c>
-      <c r="C8" s="83" t="inlineStr"/>
+      <c r="C8" s="85" t="inlineStr">
+        <is>
+          <t>— (افتراض Claude 2026-10-07 — عدّله لو مختلف)</t>
+        </is>
+      </c>
       <c r="D8" s="82" t="inlineStr">
         <is>
           <t>آخر الشهر كاش</t>
@@ -9795,7 +9932,7 @@
       </c>
       <c r="E8" s="82" t="inlineStr">
         <is>
-          <t>ناقص</t>
+          <t>محتاج مراجعة</t>
         </is>
       </c>
     </row>
@@ -9810,7 +9947,11 @@
           <t>لو حجز مدفوع اتلغى، الفلوس بترجع للعميل إزاي ومين يعتمد؟</t>
         </is>
       </c>
-      <c r="C9" s="83" t="inlineStr"/>
+      <c r="C9" s="85" t="inlineStr">
+        <is>
+          <t>الفلوس بترجع كاش من المكتب أو بنفس طريقة الدفع، بعد موافقة المدير، حسب سياسة الإلغاء (نسبة من المبلغ المحصّل) (افتراض Claude 2026-10-07 — عدّله لو مختلف)</t>
+        </is>
+      </c>
       <c r="D9" s="82" t="inlineStr">
         <is>
           <t>كاش من المكتب بعد اعتماد محمد</t>
@@ -9818,7 +9959,7 @@
       </c>
       <c r="E9" s="82" t="inlineStr">
         <is>
-          <t>ناقص</t>
+          <t>محتاج مراجعة</t>
         </is>
       </c>
     </row>
@@ -9833,7 +9974,11 @@
           <t>فيه خزنة/درج كاش في المكتب بيتقفل آخر اليوم؟ مين مسؤول عنه؟</t>
         </is>
       </c>
-      <c r="C10" s="83" t="inlineStr"/>
+      <c r="C10" s="85" t="inlineStr">
+        <is>
+          <t>خزنة المكتب بتتقفل آخر كل يوم: موظف الاستقبال يعدّ ويسلّم للمدير، والسيستم يقارن العدّ بالمسجّل (افتراض Claude 2026-10-07 — عدّله لو مختلف)</t>
+        </is>
+      </c>
       <c r="D10" s="82" t="inlineStr">
         <is>
           <t>موظف الاستقبال + تسليم يومي</t>
@@ -9841,7 +9986,7 @@
       </c>
       <c r="E10" s="82" t="inlineStr">
         <is>
-          <t>ناقص</t>
+          <t>محتاج مراجعة</t>
         </is>
       </c>
     </row>
@@ -9881,7 +10026,8 @@
     <row r="1" ht="48" customHeight="1">
       <c r="A1" s="80" t="inlineStr">
         <is>
-          <t>المصاريف اللي بتدفعها انت على كل رحلة غير المورد (رسوم دخول، مرشد، أكل، مية…). سيب الخانة فاضية لو مش موجودة.</t>
+          <t>المصاريف اللي بتدفعها انت على كل رحلة غير المورد (رسوم دخول، مرشد، أكل، مية…). سيب الخانة فاضية لو مش موجودة.
+افتراض Claude (2026-10-07): العمود «رسوم دخول» اتقرا كتكلفة تشغيل إضافية للفرد علينا، والسيستم بيحسبها جنب سعر المورد؛ عدّلها لو المعنى مختلف.</t>
         </is>
       </c>
     </row>

</xml_diff>